<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-28 16:21:17)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -10176,6 +10176,21 @@
           <t>12.05.1992</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>UM+1174926</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>29-maktab</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="T86" t="inlineStr">
         <is>
           <t>91-957-18-58</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 11:12:39)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y179"/>
+  <dimension ref="A1:Y180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -5817,6 +5817,11 @@
           <t>26-03</t>
         </is>
       </c>
+      <c r="Y47" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -10303,7 +10308,7 @@
       </c>
       <c r="Y87" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -10408,7 +10413,7 @@
       </c>
       <c r="Y88" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -10513,7 +10518,7 @@
       </c>
       <c r="Y89" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -13374,7 +13379,7 @@
       </c>
       <c r="Y114" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -16916,6 +16921,11 @@
           <t>26-04</t>
         </is>
       </c>
+      <c r="Y145" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -18860,6 +18870,11 @@
           <t>26-04</t>
         </is>
       </c>
+      <c r="Y162" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -20593,6 +20608,11 @@
           <t>26-06</t>
         </is>
       </c>
+      <c r="Y177" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -20683,6 +20703,11 @@
           <t>26-06</t>
         </is>
       </c>
+      <c r="Y178" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -20771,6 +20796,81 @@
       <c r="W179" t="inlineStr">
         <is>
           <t>26-03</t>
+        </is>
+      </c>
+      <c r="Y179" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Qulmatova Shabbona</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>29.09.2026</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Qulmatova Shabbona</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>Yo'q</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr"/>
+      <c r="P180" t="inlineStr"/>
+      <c r="Q180" t="inlineStr"/>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T180" t="inlineStr"/>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W180" t="inlineStr">
+        <is>
+          <t>26-02</t>
+        </is>
+      </c>
+      <c r="Y180" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 11:15:12)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -20823,30 +20823,21 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr">
         <is>
           <t>29.09.2026</t>
         </is>
       </c>
-      <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr">
         <is>
           <t>Qulmatova Shabbona</t>
         </is>
       </c>
-      <c r="J180" t="inlineStr"/>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
-      <c r="M180" t="inlineStr"/>
       <c r="N180" t="inlineStr">
         <is>
           <t>Yo'q</t>
         </is>
       </c>
-      <c r="O180" t="inlineStr"/>
-      <c r="P180" t="inlineStr"/>
-      <c r="Q180" t="inlineStr"/>
       <c r="R180" t="inlineStr">
         <is>
           <t>Shahodatnoma</t>
@@ -20857,7 +20848,11 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="T180" t="inlineStr"/>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>778338272</t>
+        </is>
+      </c>
       <c r="U180" t="inlineStr">
         <is>
           <t>TOPILDI</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 11:16:58)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -20828,14 +20828,49 @@
           <t>29.09.2026</t>
         </is>
       </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Azamat+qizi</t>
+        </is>
+      </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Qulmatova Shabbona</t>
+          <t>Qulmatova Shabbona Azamat+qizi</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>AE+4905104</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>61008085680019</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>05.11.2025</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>10.08.2008</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
         <is>
           <t>Yo'q</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>UM+03730102</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>70-maktab</t>
         </is>
       </c>
       <c r="R180" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 11:24:01)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -10183,7 +10183,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>UM+1174926</t>
+          <t>UM 1174926</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -20830,17 +20830,17 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Azamat+qizi</t>
+          <t>Azamat qizi</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Qulmatova Shabbona Azamat+qizi</t>
+          <t>Qulmatova Shabbona Azamat qizi</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>AE+4905104</t>
+          <t>AE4905104</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -20865,7 +20865,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>UM+03730102</t>
+          <t>UM 03730102</t>
         </is>
       </c>
       <c r="Q180" t="inlineStr">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 12:09:23)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y180"/>
+  <dimension ref="A1:Y181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20901,6 +20901,92 @@
       <c r="Y180" t="inlineStr">
         <is>
           <t>KUTILMOQDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Irgasheva Dinora</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Shodmon qizi</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Irgasheva Dinora Shodmon qizi</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>AC 2430931</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>60106035590029</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>15.11.2019</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>01.06.2003</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>UM 0441030</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr"/>
+      <c r="Q181" t="inlineStr"/>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T181" t="inlineStr"/>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V181" t="inlineStr">
+        <is>
+          <t>AI orqali tahlil qilinib qo'shildi</t>
+        </is>
+      </c>
+      <c r="W181" t="inlineStr">
+        <is>
+          <t>26-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 12:16:15)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y181"/>
+  <dimension ref="A1:Y182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20923,8 +20923,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr"/>
       <c r="G181" t="inlineStr">
         <is>
           <t>Shodmon qizi</t>
@@ -20955,14 +20953,11 @@
           <t>01.06.2003</t>
         </is>
       </c>
-      <c r="N181" t="inlineStr"/>
       <c r="O181" t="inlineStr">
         <is>
           <t>UM 0441030</t>
         </is>
       </c>
-      <c r="P181" t="inlineStr"/>
-      <c r="Q181" t="inlineStr"/>
       <c r="R181" t="inlineStr">
         <is>
           <t>Umumiy o'rta maktab</t>
@@ -20973,7 +20968,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="T181" t="inlineStr"/>
       <c r="U181" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -20985,6 +20979,96 @@
         </is>
       </c>
       <c r="W181" t="inlineStr">
+        <is>
+          <t>26-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Shonazarova Vazira</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Botir qizi</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Shonazarova Vazira Botir qizi</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>AE 4233482</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>61311085680032</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>17.09.2025</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>13.11.2008</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>UM 03730412</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr"/>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>78-maktab</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T182" t="inlineStr"/>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V182" t="inlineStr">
+        <is>
+          <t>AI orqali tahlil qilinib qo'shildi</t>
+        </is>
+      </c>
+      <c r="W182" t="inlineStr">
         <is>
           <t>26-02</t>
         </is>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 12:39:35)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -20958,6 +20958,11 @@
           <t>UM 0441030</t>
         </is>
       </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>14-maktab</t>
+        </is>
+      </c>
       <c r="R181" t="inlineStr">
         <is>
           <t>Umumiy o'rta maktab</t>
@@ -21003,8 +21008,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
-      <c r="F182" t="inlineStr"/>
       <c r="G182" t="inlineStr">
         <is>
           <t>Botir qizi</t>
@@ -21035,13 +21038,11 @@
           <t>13.11.2008</t>
         </is>
       </c>
-      <c r="N182" t="inlineStr"/>
       <c r="O182" t="inlineStr">
         <is>
           <t>UM 03730412</t>
         </is>
       </c>
-      <c r="P182" t="inlineStr"/>
       <c r="Q182" t="inlineStr">
         <is>
           <t>78-maktab</t>
@@ -21057,7 +21058,6 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="T182" t="inlineStr"/>
       <c r="U182" t="inlineStr">
         <is>
           <t>TOPILDI</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 12:53:13)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y182"/>
+  <dimension ref="A1:Y183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21069,6 +21069,104 @@
         </is>
       </c>
       <c r="W182" t="inlineStr">
+        <is>
+          <t>26-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Samatova Oydin</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Sulaymon qizi</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Samatova Oydin Sulaymon qizi</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>AD8980430</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>42910905720012</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>11.10.2024</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>29.10.1990</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>OR-SH 0346677</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr"/>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>Chiroqchi tuman 1-sonli ixtisoslashtirilgan maktab-internati</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>91-219-20-99</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V183" t="inlineStr">
+        <is>
+          <t>AI orqali tahlil qilinib qo'shildi</t>
+        </is>
+      </c>
+      <c r="W183" t="inlineStr">
         <is>
           <t>26-02</t>
         </is>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 13:00:30)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -20985,7 +20985,7 @@
       </c>
       <c r="W181" t="inlineStr">
         <is>
-          <t>26-02</t>
+          <t>26-06</t>
         </is>
       </c>
     </row>
@@ -21098,7 +21098,6 @@
           <t>146</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
           <t>Sulaymon qizi</t>
@@ -21129,13 +21128,11 @@
           <t>29.10.1990</t>
         </is>
       </c>
-      <c r="N183" t="inlineStr"/>
       <c r="O183" t="inlineStr">
         <is>
           <t>OR-SH 0346677</t>
         </is>
       </c>
-      <c r="P183" t="inlineStr"/>
       <c r="Q183" t="inlineStr">
         <is>
           <t>Chiroqchi tuman 1-sonli ixtisoslashtirilgan maktab-internati</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 13:55:44)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y183"/>
+  <dimension ref="A1:Y184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21164,6 +21164,100 @@
         </is>
       </c>
       <c r="W183" t="inlineStr">
+        <is>
+          <t>26-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Nurillayeva Dilsuz</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>326</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Mashrabovna</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Nurillayeva Dilsuz Mashrabovna</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>AD4774693</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>42506912640010</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>05.10.2023</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>25.06.1991</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>K 1607691</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr"/>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Kitob iqtisodiyot kasb-hunar kolleji</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="T184" t="inlineStr"/>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V184" t="inlineStr">
+        <is>
+          <t>AI orqali tahlil qilinib qo'shildi</t>
+        </is>
+      </c>
+      <c r="W184" t="inlineStr">
         <is>
           <t>26-02</t>
         </is>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 15:20:28)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y184"/>
+  <dimension ref="A1:AA236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,16 @@
           <t>Operator Tasdig'i</t>
         </is>
       </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Buyruq raqami</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Buyruq sanasi</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -21193,7 +21203,6 @@
           <t>326</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
           <t>Mashrabovna</t>
@@ -21224,13 +21233,11 @@
           <t>25.06.1991</t>
         </is>
       </c>
-      <c r="N184" t="inlineStr"/>
       <c r="O184" t="inlineStr">
         <is>
           <t>K 1607691</t>
         </is>
       </c>
-      <c r="P184" t="inlineStr"/>
       <c r="Q184" t="inlineStr">
         <is>
           <t>Kitob iqtisodiyot kasb-hunar kolleji</t>
@@ -21246,7 +21253,6 @@
           <t>2010</t>
         </is>
       </c>
-      <c r="T184" t="inlineStr"/>
       <c r="U184" t="inlineStr">
         <is>
           <t>TOPILDI</t>
@@ -21260,6 +21266,4146 @@
       <c r="W184" t="inlineStr">
         <is>
           <t>26-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Abdixakimova Xurshida</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Abdixakim qizi</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Abdixakimova Xurshida Abdixakim qizi</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>AD2941659</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>60409065590039</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>04.04.2023</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>04.09.2006</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>UM 02174088</t>
+        </is>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>37-maktab</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>913200125 / 914581809</t>
+        </is>
+      </c>
+      <c r="V185" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 24-11</t>
+        </is>
+      </c>
+      <c r="W185" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y185" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z185" t="inlineStr">
+        <is>
+          <t>T-47</t>
+        </is>
+      </c>
+      <c r="AA185" t="inlineStr">
+        <is>
+          <t>15.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Abdukarimova Nafosat</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Faxriddin qizi</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Abdukarimova Nafosat Faxriddin qizi</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>AD9031421</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>60205075590070</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>16.10.2024</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>02.05.2007</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>UM 03297283</t>
+        </is>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>18-maktab</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>906881531</t>
+        </is>
+      </c>
+      <c r="V186" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-22</t>
+        </is>
+      </c>
+      <c r="W186" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y186" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z186" t="inlineStr">
+        <is>
+          <t>T-29</t>
+        </is>
+      </c>
+      <c r="AA186" t="inlineStr">
+        <is>
+          <t>25.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Abduvaliyeva Jasmina</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Erkin qizi</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Abduvaliyeva Jasmina Erkin qizi</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>AD8057487</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>61311075590048</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>30.07.2024</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>13.11.2007</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>UM 03452908</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>29-sonli ayrim fanlar chuqurlashtirilgan maktab</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>779992813</t>
+        </is>
+      </c>
+      <c r="V187" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-23</t>
+        </is>
+      </c>
+      <c r="W187" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y187" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z187" t="inlineStr">
+        <is>
+          <t>T-30/1</t>
+        </is>
+      </c>
+      <c r="AA187" t="inlineStr">
+        <is>
+          <t>17.04.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Azizova Asila</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Bahodirxon qizi</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Azizova Asila Bahodirxon qizi</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>AE3401779</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>42412955590060</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>15.07.2025</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>24.12.1995</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>K 4626563</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>Shahrisabz iqtisodiyot kolleji</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>919582758</t>
+        </is>
+      </c>
+      <c r="V188" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-19</t>
+        </is>
+      </c>
+      <c r="W188" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y188" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z188" t="inlineStr">
+        <is>
+          <t>T-32</t>
+        </is>
+      </c>
+      <c r="AA188" t="inlineStr">
+        <is>
+          <t>14.05.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Baxtiyorova Dinora</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Akmal qizi</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Baxtiyorova Dinora Akmal qizi</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>AD7645847</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>62307075680084</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>27.06.2024</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>23.07.2007</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>PT 0017689</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>2-sonli politexnikum</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T189" t="inlineStr"/>
+      <c r="V189" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-18</t>
+        </is>
+      </c>
+      <c r="W189" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y189" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z189" t="inlineStr">
+        <is>
+          <t>T-26</t>
+        </is>
+      </c>
+      <c r="AA189" t="inlineStr">
+        <is>
+          <t>12.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Mahmudjonova Mohinur</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Sanjar qizi</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Mahmudjonova Mohinur Sanjar qizi</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>AD4538974</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>62504065680035</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>08.09.2023</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>25.04.2006</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>UM 02289977</t>
+        </is>
+      </c>
+      <c r="Q190" t="inlineStr">
+        <is>
+          <t>290-maktab</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr"/>
+      <c r="V190" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-23</t>
+        </is>
+      </c>
+      <c r="W190" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y190" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z190" t="inlineStr">
+        <is>
+          <t>T-45</t>
+        </is>
+      </c>
+      <c r="AA190" t="inlineStr">
+        <is>
+          <t>22.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Mahmudova Vasila</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Hujjat qizi</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Mahmudova Vasila Hujjat qizi</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>AD9687160</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>62206075680112</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>04.12.2024</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>22.06.2007</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>UM 03275718</t>
+        </is>
+      </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>81-maktab</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T191" t="inlineStr"/>
+      <c r="V191" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-17</t>
+        </is>
+      </c>
+      <c r="W191" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y191" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z191" t="inlineStr">
+        <is>
+          <t>T-36</t>
+        </is>
+      </c>
+      <c r="AA191" t="inlineStr">
+        <is>
+          <t>01.06.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Nasimova Durdona</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Yormahmat qizi</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Nasimova Durdona Yormahmat qizi</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>62605065680039</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>26.05.2006</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr"/>
+      <c r="Q192" t="inlineStr"/>
+      <c r="R192" t="inlineStr"/>
+      <c r="T192" t="inlineStr"/>
+      <c r="V192" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 201 (24-11)</t>
+        </is>
+      </c>
+      <c r="W192" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y192" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z192" t="inlineStr">
+        <is>
+          <t>T-06</t>
+        </is>
+      </c>
+      <c r="AA192" t="inlineStr">
+        <is>
+          <t>28.10.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Nishonova Hilola</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Faxriddin qizi</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Nishonova Hilola Faxriddin qizi</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>AD2578567</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>60205055720048</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>14.02.2023</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>02.05.2005</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>UM 01890968</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>24-maktab</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>914662205</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-19</t>
+        </is>
+      </c>
+      <c r="W193" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y193" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z193" t="inlineStr">
+        <is>
+          <t>T-33</t>
+        </is>
+      </c>
+      <c r="AA193" t="inlineStr">
+        <is>
+          <t>14.05.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Nomazova Rayhona</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Murodullo qizi</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Nomazova Rayhona Murodullo qizi</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>AD9665620</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>62702075630033</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>03.12.2024</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>27.02.2007</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>UM 03287195</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>70-maktab</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T194" t="inlineStr"/>
+      <c r="V194" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-17</t>
+        </is>
+      </c>
+      <c r="W194" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y194" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z194" t="inlineStr">
+        <is>
+          <t>T-44</t>
+        </is>
+      </c>
+      <c r="AA194" t="inlineStr">
+        <is>
+          <t>07.09.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Norboboyeva Zahro</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Nuriddin qizi</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Norboboyeva Zahro Nuriddin qizi</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>61107075680027</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>11.07.2007</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr"/>
+      <c r="Q195" t="inlineStr"/>
+      <c r="R195" t="inlineStr"/>
+      <c r="T195" t="inlineStr"/>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 203 (24-13)</t>
+        </is>
+      </c>
+      <c r="W195" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y195" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z195" t="inlineStr">
+        <is>
+          <t>T-11</t>
+        </is>
+      </c>
+      <c r="AA195" t="inlineStr">
+        <is>
+          <t>29.11.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Omonova Dilorom</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Toshkent qizi</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Omonova Dilorom Toshkent qizi</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr"/>
+      <c r="L196" t="inlineStr"/>
+      <c r="M196" t="inlineStr"/>
+      <c r="O196" t="inlineStr"/>
+      <c r="Q196" t="inlineStr"/>
+      <c r="R196" t="inlineStr"/>
+      <c r="T196" t="inlineStr"/>
+      <c r="V196" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 24-12</t>
+        </is>
+      </c>
+      <c r="W196" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y196" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z196" t="inlineStr">
+        <is>
+          <t>T-20</t>
+        </is>
+      </c>
+      <c r="AA196" t="inlineStr">
+        <is>
+          <t>23.02.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Otaqulova Moxiniso</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Tursunpo'lat qizi</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Otaqulova Moxiniso Tursunpo'lat qizi</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>60703055720061</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr"/>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>07.03.2005</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr"/>
+      <c r="Q197" t="inlineStr"/>
+      <c r="R197" t="inlineStr"/>
+      <c r="T197" t="inlineStr"/>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 201 (24-11)</t>
+        </is>
+      </c>
+      <c r="W197" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y197" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z197" t="inlineStr">
+        <is>
+          <t>T-07</t>
+        </is>
+      </c>
+      <c r="AA197" t="inlineStr">
+        <is>
+          <t>28.10.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Qurbonova Gulida</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Xusan qizi</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Qurbonova Gulida Xusan qizi</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>AB3682339</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>41207975590067</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>07.04.2016</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>12.07.1997</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>K 4165742</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>2-Shahrisabz xizmat ko'rsatish kolleji</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>886949700</t>
+        </is>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-20</t>
+        </is>
+      </c>
+      <c r="W198" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y198" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z198" t="inlineStr">
+        <is>
+          <t>T-35</t>
+        </is>
+      </c>
+      <c r="AA198" t="inlineStr">
+        <is>
+          <t>18.05.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Raimova Zulfizar</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Rasulovna</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Raimova Zulfizar Rasulovna</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>AD4408617</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>41007872560088</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>10.07.1987</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>10.07.1987</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>K 5489037</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>Yakkabog' qurulish sanoat kolleji</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T199" t="inlineStr"/>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-16</t>
+        </is>
+      </c>
+      <c r="W199" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y199" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z199" t="inlineStr">
+        <is>
+          <t>T-34</t>
+        </is>
+      </c>
+      <c r="AA199" t="inlineStr">
+        <is>
+          <t>15.05.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Sayfilloyeva Anisa</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Jamshidzoda</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Sayfilloyeva Anisa Jamshidzoda</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>AD8565644</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>61908085680094</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>10.09.2024</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>19.08.2008</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>UM 03275869</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>89-maktab</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T200" t="inlineStr"/>
+      <c r="V200" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-23</t>
+        </is>
+      </c>
+      <c r="W200" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y200" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z200" t="inlineStr">
+        <is>
+          <t>T-22</t>
+        </is>
+      </c>
+      <c r="AA200" t="inlineStr">
+        <is>
+          <t>25.02.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Sayfiyeva Parizod</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Zafarovna</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Sayfiyeva Parizod Zafarovna</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>AD2082802</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>60601065680048</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>25.11.2022</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>06.01.2006</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>UM 02151494</t>
+        </is>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>53-maktab</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T201" t="inlineStr"/>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-21</t>
+        </is>
+      </c>
+      <c r="W201" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y201" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z201" t="inlineStr"/>
+      <c r="AA201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Sayfullayeva Kumush</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Lutfullo qizi</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Sayfullayeva Kumush Lutfullo qizi</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>AD1789847</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>62009055680038</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>22.09.2022</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>20.09.2005</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>UM 01903229</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>82-maktab</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>887040920 / 975878105</t>
+        </is>
+      </c>
+      <c r="V202" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 24-13</t>
+        </is>
+      </c>
+      <c r="W202" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y202" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z202" t="inlineStr">
+        <is>
+          <t>T-30</t>
+        </is>
+      </c>
+      <c r="AA202" t="inlineStr">
+        <is>
+          <t>14.04.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Shodiyeva Fayyoza</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Farxod qizi</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Shodiyeva Fayyoza Farxod qizi</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr"/>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>60706065590040</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr"/>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>07.06.2006</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr"/>
+      <c r="Q203" t="inlineStr"/>
+      <c r="R203" t="inlineStr"/>
+      <c r="T203" t="inlineStr"/>
+      <c r="V203" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 204 (24-14)</t>
+        </is>
+      </c>
+      <c r="W203" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y203" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z203" t="inlineStr"/>
+      <c r="AA203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>To'rayeva Elsenora</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Sobir qizi</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>To'rayeva Elsenora Sobir qizi</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr"/>
+      <c r="K204" t="inlineStr"/>
+      <c r="L204" t="inlineStr"/>
+      <c r="M204" t="inlineStr"/>
+      <c r="O204" t="inlineStr"/>
+      <c r="Q204" t="inlineStr"/>
+      <c r="R204" t="inlineStr"/>
+      <c r="T204" t="inlineStr"/>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 24-12</t>
+        </is>
+      </c>
+      <c r="W204" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y204" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z204" t="inlineStr">
+        <is>
+          <t>T-21</t>
+        </is>
+      </c>
+      <c r="AA204" t="inlineStr">
+        <is>
+          <t>23.02.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Uroqova Muslima</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Anvar qizi</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Uroqova Muslima Anvar qizi</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>AD6021065</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>61611065720061</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>05.02.2024</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>16.11.2006</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>UM 02140025</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>24-maktab</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>919579806 / 906750477</t>
+        </is>
+      </c>
+      <c r="V205" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 24-14</t>
+        </is>
+      </c>
+      <c r="W205" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y205" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z205" t="inlineStr"/>
+      <c r="AA205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Usmonjonova Marjona</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Dilshod qizi</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Usmonjonova Marjona Dilshod qizi</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>AC0170536</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>61605025680021</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>09.11.2018</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>16.05.2002</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>D 0098091</t>
+        </is>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>Qishloq xo'jalik kolleji</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>884901605 / 908787811</t>
+        </is>
+      </c>
+      <c r="V206" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 24-12</t>
+        </is>
+      </c>
+      <c r="W206" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y206" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z206" t="inlineStr"/>
+      <c r="AA206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Xusanboyeva Fotimaxon</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Baxtiyor qizi</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Xusanboyeva Fotimaxon Baxtiyor qizi</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>AD4614901</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>60805045930053</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>15.09.2023</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>08.05.2004</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>UM 1347858</t>
+        </is>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>22-maktab</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T207" t="inlineStr"/>
+      <c r="V207" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-23</t>
+        </is>
+      </c>
+      <c r="W207" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y207" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z207" t="inlineStr">
+        <is>
+          <t>T-30/2</t>
+        </is>
+      </c>
+      <c r="AA207" t="inlineStr">
+        <is>
+          <t>17.04.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Yusupova Asila</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Iskandar qizi</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Yusupova Asila Iskandar qizi</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>AD0311873</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>61007015680048</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>13.04.2021</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>10.07.2001</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>UM 0085864</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>51-maktab</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T208" t="inlineStr"/>
+      <c r="V208" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-20</t>
+        </is>
+      </c>
+      <c r="W208" t="inlineStr">
+        <is>
+          <t>Akademik ta'til olganlar</t>
+        </is>
+      </c>
+      <c r="Y208" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z208" t="inlineStr">
+        <is>
+          <t>T-25</t>
+        </is>
+      </c>
+      <c r="AA208" t="inlineStr">
+        <is>
+          <t>10.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Abdialimova Nilufar</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Akbar qizi</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Abdialimova Nilufar Akbar qizi</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>AD0968690</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>60908045720047</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>07.01.2022</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>09.08.2004</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>UM 1306544</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>3-maktab</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T209" t="inlineStr"/>
+      <c r="V209" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 25-16</t>
+        </is>
+      </c>
+      <c r="W209" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y209" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z209" t="inlineStr">
+        <is>
+          <t>T-23</t>
+        </is>
+      </c>
+      <c r="AA209" t="inlineStr">
+        <is>
+          <t>02.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Baxtiyorova Fotima</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Zarif qizi</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Baxtiyorova Fotima Zarif qizi</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>AD9120079</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>60510075680079</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>23.10.2024</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>05.10.2007</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>UM 03273958</t>
+        </is>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>22-maktab</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T210" t="inlineStr"/>
+      <c r="V210" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W210" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y210" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z210" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA210" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>G'abborova Xosiyat</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Nosir qizi</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>G'abborova Xosiyat Nosir qizi</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>AD8770653</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>61011065630054</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>25.09.2024</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>10.11.2006</t>
+        </is>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>UM 03287373</t>
+        </is>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>78-maktab</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>974295606</t>
+        </is>
+      </c>
+      <c r="V211" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W211" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y211" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z211" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA211" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Hasanova Gulsevar</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Lochinbek qizi</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Hasanova Gulsevar Lochinbek qizi</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr"/>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>61204065730042</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr"/>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>12.04.2006</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr"/>
+      <c r="Q212" t="inlineStr"/>
+      <c r="R212" t="inlineStr"/>
+      <c r="T212" t="inlineStr"/>
+      <c r="V212" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 202 (24-12)</t>
+        </is>
+      </c>
+      <c r="W212" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y212" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z212" t="inlineStr">
+        <is>
+          <t>T-09</t>
+        </is>
+      </c>
+      <c r="AA212" t="inlineStr">
+        <is>
+          <t>30.10.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Jabborova Anora</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Nuriddin qizi</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Jabborova Anora Nuriddin qizi</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>AD8537425</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>62009075720031</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>09.09.2024</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>20.09.2007</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>UM 03264707</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>58-maktab</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr"/>
+      <c r="V213" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-23</t>
+        </is>
+      </c>
+      <c r="W213" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y213" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z213" t="inlineStr">
+        <is>
+          <t>T-37</t>
+        </is>
+      </c>
+      <c r="AA213" t="inlineStr">
+        <is>
+          <t>08.07.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Jumanova Xolinisa</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Orif qizi</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Jumanova Xolinisa Orif qizi</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>AD9356181</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>60904075730067</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>11.11.2024</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>09.04.2007</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>UM 03300691</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>50-maktab</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>957022572</t>
+        </is>
+      </c>
+      <c r="V214" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-17</t>
+        </is>
+      </c>
+      <c r="W214" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y214" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z214" t="inlineStr">
+        <is>
+          <t>T-40</t>
+        </is>
+      </c>
+      <c r="AA214" t="inlineStr">
+        <is>
+          <t>26.08.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Jumayeva Xurshida</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Safar qizi</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>Jumayeva Xurshida Safar qizi</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr"/>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>61201045630052</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr"/>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>12.01.2004</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr"/>
+      <c r="Q215" t="inlineStr"/>
+      <c r="R215" t="inlineStr"/>
+      <c r="T215" t="inlineStr"/>
+      <c r="V215" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 204 (24-14)</t>
+        </is>
+      </c>
+      <c r="W215" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y215" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z215" t="inlineStr"/>
+      <c r="AA215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Mahmudova Munisa</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Mahsudjonovna</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Mahmudova Munisa Mahsudjonovna</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr"/>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>62206055590013</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr"/>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>22.06.2005</t>
+        </is>
+      </c>
+      <c r="O216" t="inlineStr"/>
+      <c r="Q216" t="inlineStr"/>
+      <c r="R216" t="inlineStr"/>
+      <c r="T216" t="inlineStr"/>
+      <c r="V216" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 205 (24-15)</t>
+        </is>
+      </c>
+      <c r="W216" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y216" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z216" t="inlineStr">
+        <is>
+          <t>T-10</t>
+        </is>
+      </c>
+      <c r="AA216" t="inlineStr">
+        <is>
+          <t>30.10.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Meyliqulova Sabrina</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Baxtiyor qizi</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>Meyliqulova Sabrina Baxtiyor qizi</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>AD8641562</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>61709075590063</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>16.09.2024</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>17.09.2007</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>UM 03296986</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>10-maktab</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr"/>
+      <c r="V217" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-16</t>
+        </is>
+      </c>
+      <c r="W217" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y217" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z217" t="inlineStr">
+        <is>
+          <t>T-24</t>
+        </is>
+      </c>
+      <c r="AA217" t="inlineStr">
+        <is>
+          <t>02.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Numonova Feruza</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Mirhomid qizi</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Numonova Feruza Mirhomid qizi</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr"/>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>62808027890020</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr"/>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>28.08.2002</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr"/>
+      <c r="Q218" t="inlineStr"/>
+      <c r="R218" t="inlineStr"/>
+      <c r="T218" t="inlineStr"/>
+      <c r="V218" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 203 (24-13)</t>
+        </is>
+      </c>
+      <c r="W218" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y218" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z218" t="inlineStr">
+        <is>
+          <t>T-05</t>
+        </is>
+      </c>
+      <c r="AA218" t="inlineStr">
+        <is>
+          <t>13.10.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Omonova Sumbula</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Farxod qizi</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>Omonova Sumbula Farxod qizi</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>AD1292785</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>60404055590037</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>23,04,2022</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr"/>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>UM 01924159</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>36-sonli ayrim fanlar chuqur o'rgatiladigan ixtisoslashtirilgan maktab</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>779845421</t>
+        </is>
+      </c>
+      <c r="V219" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W219" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y219" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z219" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA219" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Qarshiyeva Ruxshona</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Otabek qizi</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>Qarshiyeva Ruxshona Otabek qizi</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>AD8751204</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>60512075590040</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>24.09.2024</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>05.12.2007</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>PT 0256788</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>1-sonli politexnikum</t>
+        </is>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>918157227</t>
+        </is>
+      </c>
+      <c r="V220" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W220" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y220" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z220" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA220" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Salimova Zarina</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Sobirjon qizi</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>Salimova Zarina Sobirjon qizi</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>AD8890500</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>42110975590034</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>07.10.2024</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>21.10.1997</t>
+        </is>
+      </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>K 4174786</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>Shahrisabz yengil sanoat va xizmat ko'rsatish kolleji</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>880019709 / 916340177</t>
+        </is>
+      </c>
+      <c r="V221" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 24-15</t>
+        </is>
+      </c>
+      <c r="W221" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y221" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z221" t="inlineStr">
+        <is>
+          <t>T-27</t>
+        </is>
+      </c>
+      <c r="AA221" t="inlineStr">
+        <is>
+          <t>18.03.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Saydaliyeva Sevinch</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Alimdjan qizi</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>Saydaliyeva Sevinch Alimdjan qizi</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>AD3193422</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>60904075590012</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>03.05.2023</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>09.04.2007</t>
+        </is>
+      </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>PT 0176960</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>Sharisabz shahar 2-sonli kasb-hunar maktabi</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>000</t>
+        </is>
+      </c>
+      <c r="V222" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-20</t>
+        </is>
+      </c>
+      <c r="W222" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y222" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z222" t="inlineStr"/>
+      <c r="AA222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Soliyeva E'zoza</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Sherbobo qizi</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>Soliyeva E'zoza Sherbobo qizi</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>AD4615905</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>61803065680094</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>15.09.2023</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>18.03.2006</t>
+        </is>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>UM 02151153</t>
+        </is>
+      </c>
+      <c r="Q223" t="inlineStr">
+        <is>
+          <t>44-maktab</t>
+        </is>
+      </c>
+      <c r="R223" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T223" t="inlineStr"/>
+      <c r="V223" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W223" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y223" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z223" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA223" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Suyunova Marjona</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Ravshan qizi</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>Suyunova Marjona Ravshan qizi</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr"/>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>60704065720162</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr"/>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>07.04.2006</t>
+        </is>
+      </c>
+      <c r="O224" t="inlineStr"/>
+      <c r="Q224" t="inlineStr"/>
+      <c r="R224" t="inlineStr"/>
+      <c r="T224" t="inlineStr"/>
+      <c r="V224" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 202 (24-12)</t>
+        </is>
+      </c>
+      <c r="W224" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y224" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z224" t="inlineStr"/>
+      <c r="AA224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Suyunova Ruxshona</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Karimjon qizi</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>Suyunova Ruxshona Karimjon qizi</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr"/>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>61405065680104</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr"/>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>14.05.2006</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr"/>
+      <c r="Q225" t="inlineStr"/>
+      <c r="R225" t="inlineStr"/>
+      <c r="T225" t="inlineStr"/>
+      <c r="V225" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs, oldingi guruh 203 (24-13)</t>
+        </is>
+      </c>
+      <c r="W225" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y225" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z225" t="inlineStr">
+        <is>
+          <t>T-12</t>
+        </is>
+      </c>
+      <c r="AA225" t="inlineStr">
+        <is>
+          <t>29.11.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Suyunova Shaxlo</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Tohir qizi</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>Suyunova Shaxlo Tohir qizi</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr"/>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>61305065720094</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr"/>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>13.05.2006</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr"/>
+      <c r="Q226" t="inlineStr"/>
+      <c r="R226" t="inlineStr"/>
+      <c r="T226" t="inlineStr"/>
+      <c r="V226" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 203 (24-13)</t>
+        </is>
+      </c>
+      <c r="W226" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y226" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z226" t="inlineStr"/>
+      <c r="AA226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>To'xtayeva Shirida</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Sirojiddin qizi</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>To'xtayeva Shirida Sirojiddin qizi</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>AD1403124</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>61906055680059</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>30.05.2022</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>19.06.2005</t>
+        </is>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>UM 1296145</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>7-maktab</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>990598714</t>
+        </is>
+      </c>
+      <c r="V227" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W227" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y227" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z227" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA227" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Toshkentova Sevinchoy</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Zayniddin qizi</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>Toshkentova Sevinchoy Zayniddin qizi</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>AD6867124</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>60505075730035</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>18.04.2024</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>05.05.2007</t>
+        </is>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>UM 03301249</t>
+        </is>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>72-maktab</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T228" t="inlineStr"/>
+      <c r="V228" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W228" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y228" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z228" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA228" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Tug'izova Zahro</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Tohir qizi</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>Tug'izova Zahro Tohir qizi</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr"/>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>62912005590041</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr"/>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>29.12.2000</t>
+        </is>
+      </c>
+      <c r="O229" t="inlineStr"/>
+      <c r="Q229" t="inlineStr"/>
+      <c r="R229" t="inlineStr"/>
+      <c r="T229" t="inlineStr"/>
+      <c r="V229" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 205 (24-15)</t>
+        </is>
+      </c>
+      <c r="W229" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y229" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z229" t="inlineStr">
+        <is>
+          <t>T-08</t>
+        </is>
+      </c>
+      <c r="AA229" t="inlineStr">
+        <is>
+          <t>30.10.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Tursunova Sevinch</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Turg'un qizi</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>Tursunova Sevinch Turg'un qizi</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr"/>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>61905075680098</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr"/>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>19.05.2007</t>
+        </is>
+      </c>
+      <c r="O230" t="inlineStr"/>
+      <c r="Q230" t="inlineStr"/>
+      <c r="R230" t="inlineStr"/>
+      <c r="T230" t="inlineStr"/>
+      <c r="V230" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 203 (24-13)</t>
+        </is>
+      </c>
+      <c r="W230" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y230" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z230" t="inlineStr"/>
+      <c r="AA230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Usmonova Jasmina</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Nodir qizi</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>Usmonova Jasmina Nodir qizi</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>AD9134105</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>62712075590017</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>24.10.2024</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>27.12.2007</t>
+        </is>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>UM 03298099</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>45-maktab</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>919603730</t>
+        </is>
+      </c>
+      <c r="V231" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 1-kurs, oldingi guruh 25-17</t>
+        </is>
+      </c>
+      <c r="W231" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y231" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z231" t="inlineStr">
+        <is>
+          <t>T-13</t>
+        </is>
+      </c>
+      <c r="AA231" t="inlineStr">
+        <is>
+          <t>16.12.2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Usmonova Shabbona</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Botir qizi</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>Usmonova Shabbona Botir qizi</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>AD9713077</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>61412075590059</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>06.12.2024</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>14.12.2007</t>
+        </is>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>UM 03295752</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>7-maktab</t>
+        </is>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>505890781</t>
+        </is>
+      </c>
+      <c r="V232" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W232" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y232" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z232" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA232" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Xamrayeva Niginabonu</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Jamshid qizi</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>Xamrayeva Niginabonu Jamshid qizi</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>AD9506052</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>61508075590121</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>21,11,2024</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr"/>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>UM 03295886</t>
+        </is>
+      </c>
+      <c r="Q233" t="inlineStr">
+        <is>
+          <t>10-maktab</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr"/>
+      <c r="V233" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W233" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y233" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z233" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA233" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Yoqubova Maftuna</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Hushvaqt qizi</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>Yoqubova Maftuna Hushvaqt qizi</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>AE2747402</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>40312902560107</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>20,05,2025</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr"/>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>K 1234480</t>
+        </is>
+      </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>Miroqi sport pedagogika kolleji</t>
+        </is>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr"/>
+      <c r="V234" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W234" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y234" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z234" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA234" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Yuldosheva Iroda</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Hasanovna</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>Yuldosheva Iroda Hasanovna</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>AB7535578</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>40108945590034</t>
+        </is>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>22,08,2017</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr"/>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>K 2404534</t>
+        </is>
+      </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>Shahrisabz pedagogika kolleji</t>
+        </is>
+      </c>
+      <c r="R235" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T235" t="inlineStr"/>
+      <c r="V235" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W235" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y235" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z235" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA235" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Ziyadullayeva Zahro</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Ubaydullo qizi</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>Ziyadullayeva Zahro Ubaydullo qizi</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>AD8888020</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>62609075590027</t>
+        </is>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>07,10,2024</t>
+        </is>
+      </c>
+      <c r="M236" t="inlineStr"/>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>UM 03295463</t>
+        </is>
+      </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>1-maktab</t>
+        </is>
+      </c>
+      <c r="R236" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="T236" t="inlineStr">
+        <is>
+          <t>972904017</t>
+        </is>
+      </c>
+      <c r="V236" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: TSCH ro`yxati (guruhi ko`rsatilmagan)</t>
+        </is>
+      </c>
+      <c r="W236" t="inlineStr">
+        <is>
+          <t>Talabalar safidan chiqarilganlar</t>
+        </is>
+      </c>
+      <c r="Y236" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="Z236" t="inlineStr">
+        <is>
+          <t>T-14/T-15</t>
+        </is>
+      </c>
+      <c r="AA236" t="inlineStr">
+        <is>
+          <t>20.01.2026/21.01.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 16:22:47)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -33093,7 +33093,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T334" t="inlineStr"/>
       <c r="V334" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -33889,7 +33888,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T344" t="inlineStr"/>
       <c r="V344" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34045,7 +34043,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T346" t="inlineStr"/>
       <c r="V346" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34121,7 +34118,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T347" t="inlineStr"/>
       <c r="V347" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34197,7 +34193,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T348" t="inlineStr"/>
       <c r="V348" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34353,7 +34348,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T350" t="inlineStr"/>
       <c r="V350" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34429,7 +34423,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T351" t="inlineStr"/>
       <c r="V351" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34505,7 +34498,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T352" t="inlineStr"/>
       <c r="V352" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34661,7 +34653,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T354" t="inlineStr"/>
       <c r="V354" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34817,7 +34808,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T356" t="inlineStr"/>
       <c r="V356" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -34893,7 +34883,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T357" t="inlineStr"/>
       <c r="V357" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -35049,7 +35038,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T359" t="inlineStr"/>
       <c r="V359" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -35125,7 +35113,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T360" t="inlineStr"/>
       <c r="V360" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -35441,7 +35428,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T364" t="inlineStr"/>
       <c r="V364" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -35597,7 +35583,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T366" t="inlineStr"/>
       <c r="V366" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -35673,7 +35658,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T367" t="inlineStr"/>
       <c r="V367" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -35829,7 +35813,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T369" t="inlineStr"/>
       <c r="V369" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -36065,7 +36048,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T372" t="inlineStr"/>
       <c r="V372" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -36301,7 +36283,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T375" t="inlineStr"/>
       <c r="V375" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -36537,7 +36518,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T378" t="inlineStr"/>
       <c r="V378" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -36613,7 +36593,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T379" t="inlineStr"/>
       <c r="V379" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -36849,7 +36828,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T382" t="inlineStr"/>
       <c r="V382" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -36925,7 +36903,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T383" t="inlineStr"/>
       <c r="V383" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -37161,7 +37138,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T386" t="inlineStr"/>
       <c r="V386" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -37317,7 +37293,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T388" t="inlineStr"/>
       <c r="V388" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -37393,7 +37368,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T389" t="inlineStr"/>
       <c r="V389" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -37469,7 +37443,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T390" t="inlineStr"/>
       <c r="V390" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -37625,7 +37598,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T392" t="inlineStr"/>
       <c r="V392" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -37781,7 +37753,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T394" t="inlineStr"/>
       <c r="V394" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -37857,7 +37828,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T395" t="inlineStr"/>
       <c r="V395" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -38253,7 +38223,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T400" t="inlineStr"/>
       <c r="V400" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -38409,7 +38378,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T402" t="inlineStr"/>
       <c r="V402" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -38485,7 +38453,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T403" t="inlineStr"/>
       <c r="V403" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -38561,7 +38528,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T404" t="inlineStr"/>
       <c r="V404" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -38877,7 +38843,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T408" t="inlineStr"/>
       <c r="V408" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -38953,7 +38918,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T409" t="inlineStr"/>
       <c r="V409" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -39109,7 +39073,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T411" t="inlineStr"/>
       <c r="V411" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -39425,7 +39388,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T415" t="inlineStr"/>
       <c r="V415" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -39581,7 +39543,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T417" t="inlineStr"/>
       <c r="V417" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -39657,7 +39618,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T418" t="inlineStr"/>
       <c r="V418" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -39733,7 +39693,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T419" t="inlineStr"/>
       <c r="V419" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -39809,7 +39768,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T420" t="inlineStr"/>
       <c r="V420" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -39965,7 +39923,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T422" t="inlineStr"/>
       <c r="V422" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -40121,7 +40078,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T424" t="inlineStr"/>
       <c r="V424" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -40277,7 +40233,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T426" t="inlineStr"/>
       <c r="V426" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -40513,7 +40468,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T429" t="inlineStr"/>
       <c r="V429" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -40669,7 +40623,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T431" t="inlineStr"/>
       <c r="V431" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -40825,7 +40778,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T433" t="inlineStr"/>
       <c r="V433" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -40981,7 +40933,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T435" t="inlineStr"/>
       <c r="V435" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -41137,7 +41088,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T437" t="inlineStr"/>
       <c r="V437" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -41293,7 +41243,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T439" t="inlineStr"/>
       <c r="V439" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -41449,7 +41398,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T441" t="inlineStr"/>
       <c r="V441" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -41525,7 +41473,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T442" t="inlineStr"/>
       <c r="V442" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -41601,7 +41548,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T443" t="inlineStr"/>
       <c r="V443" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -43037,7 +42983,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T461" t="inlineStr"/>
       <c r="V461" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -43273,7 +43218,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T464" t="inlineStr"/>
       <c r="V464" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -43349,7 +43293,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T465" t="inlineStr"/>
       <c r="V465" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -43425,7 +43368,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T466" t="inlineStr"/>
       <c r="V466" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -43741,7 +43683,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T470" t="inlineStr"/>
       <c r="V470" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44057,7 +43998,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T474" t="inlineStr"/>
       <c r="V474" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44133,7 +44073,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T475" t="inlineStr"/>
       <c r="V475" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44194,10 +44133,6 @@
           <t>27.04.1997</t>
         </is>
       </c>
-      <c r="O476" t="inlineStr"/>
-      <c r="Q476" t="inlineStr"/>
-      <c r="R476" t="inlineStr"/>
-      <c r="T476" t="inlineStr"/>
       <c r="V476" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44353,7 +44288,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T478" t="inlineStr"/>
       <c r="V478" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44429,7 +44363,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T479" t="inlineStr"/>
       <c r="V479" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44505,7 +44438,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T480" t="inlineStr"/>
       <c r="V480" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44581,7 +44513,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T481" t="inlineStr"/>
       <c r="V481" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44624,7 +44555,7 @@
       </c>
       <c r="J482" t="inlineStr">
         <is>
-          <t>AB6959079</t>
+          <t>AD 4323840</t>
         </is>
       </c>
       <c r="K482" t="inlineStr">
@@ -44657,7 +44588,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T482" t="inlineStr"/>
       <c r="V482" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44733,7 +44663,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T483" t="inlineStr"/>
       <c r="V483" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44889,7 +44818,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T485" t="inlineStr"/>
       <c r="V485" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44965,7 +44893,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T486" t="inlineStr"/>
       <c r="V486" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45026,10 +44953,6 @@
           <t>31.01.1996</t>
         </is>
       </c>
-      <c r="O487" t="inlineStr"/>
-      <c r="Q487" t="inlineStr"/>
-      <c r="R487" t="inlineStr"/>
-      <c r="T487" t="inlineStr"/>
       <c r="V487" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45105,7 +45028,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T488" t="inlineStr"/>
       <c r="V488" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45341,7 +45263,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T491" t="inlineStr"/>
       <c r="V491" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45497,7 +45418,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T493" t="inlineStr"/>
       <c r="V493" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45573,7 +45493,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T494" t="inlineStr"/>
       <c r="V494" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45649,7 +45568,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T495" t="inlineStr"/>
       <c r="V495" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45805,7 +45723,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T497" t="inlineStr"/>
       <c r="V497" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45961,7 +45878,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T499" t="inlineStr"/>
       <c r="V499" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -46117,7 +46033,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T501" t="inlineStr"/>
       <c r="V501" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -46513,7 +46428,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T506" t="inlineStr"/>
       <c r="V506" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -46589,7 +46503,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T507" t="inlineStr"/>
       <c r="V507" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -46665,7 +46578,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T508" t="inlineStr"/>
       <c r="V508" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -46741,7 +46653,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T509" t="inlineStr"/>
       <c r="V509" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -47057,7 +46968,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T513" t="inlineStr"/>
       <c r="V513" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -47133,7 +47043,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T514" t="inlineStr"/>
       <c r="V514" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -47289,7 +47198,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T516" t="inlineStr"/>
       <c r="V516" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -47605,7 +47513,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T520" t="inlineStr"/>
       <c r="V520" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -47761,7 +47668,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T522" t="inlineStr"/>
       <c r="V522" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -47917,7 +47823,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T524" t="inlineStr"/>
       <c r="V524" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48153,7 +48058,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T527" t="inlineStr"/>
       <c r="V527" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48219,7 +48123,6 @@
           <t>IM 000125</t>
         </is>
       </c>
-      <c r="Q528" t="inlineStr"/>
       <c r="R528" t="inlineStr">
         <is>
           <t>Umumiy o'rta maktab</t>
@@ -48305,7 +48208,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T529" t="inlineStr"/>
       <c r="V529" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48381,7 +48283,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T530" t="inlineStr"/>
       <c r="V530" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48457,7 +48358,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T531" t="inlineStr"/>
       <c r="V531" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48533,7 +48433,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T532" t="inlineStr"/>
       <c r="V532" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48609,7 +48508,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T533" t="inlineStr"/>
       <c r="V533" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48685,7 +48583,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T534" t="inlineStr"/>
       <c r="V534" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48761,7 +48658,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T535" t="inlineStr"/>
       <c r="V535" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48837,7 +48733,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T536" t="inlineStr"/>
       <c r="V536" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48913,7 +48808,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T537" t="inlineStr"/>
       <c r="V537" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48989,7 +48883,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T538" t="inlineStr"/>
       <c r="V538" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49065,7 +48958,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T539" t="inlineStr"/>
       <c r="V539" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49141,7 +49033,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T540" t="inlineStr"/>
       <c r="V540" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49202,10 +49093,6 @@
           <t>20.03.2002</t>
         </is>
       </c>
-      <c r="O541" t="inlineStr"/>
-      <c r="Q541" t="inlineStr"/>
-      <c r="R541" t="inlineStr"/>
-      <c r="T541" t="inlineStr"/>
       <c r="V541" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49281,7 +49168,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T542" t="inlineStr"/>
       <c r="V542" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49357,7 +49243,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T543" t="inlineStr"/>
       <c r="V543" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49433,7 +49318,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T544" t="inlineStr"/>
       <c r="V544" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49509,7 +49393,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T545" t="inlineStr"/>
       <c r="V545" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49665,7 +49548,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T547" t="inlineStr"/>
       <c r="V547" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49741,7 +49623,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T548" t="inlineStr"/>
       <c r="V548" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49882,10 +49763,6 @@
           <t>19.07.1995</t>
         </is>
       </c>
-      <c r="O550" t="inlineStr"/>
-      <c r="Q550" t="inlineStr"/>
-      <c r="R550" t="inlineStr"/>
-      <c r="T550" t="inlineStr"/>
       <c r="V550" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -50041,7 +49918,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T552" t="inlineStr"/>
       <c r="V552" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -50117,7 +49993,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T553" t="inlineStr"/>
       <c r="V553" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -50353,7 +50228,6 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
-      <c r="T556" t="inlineStr"/>
       <c r="V556" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -50429,7 +50303,6 @@
           <t>Kollej</t>
         </is>
       </c>
-      <c r="T557" t="inlineStr"/>
       <c r="V557" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 16:24:11)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -8866,7 +8866,7 @@
       </c>
       <c r="Y74" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -21345,7 +21345,7 @@
       </c>
       <c r="Y185" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z185" t="inlineStr">
@@ -21435,7 +21435,7 @@
       </c>
       <c r="Y186" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z186" t="inlineStr">
@@ -21525,7 +21525,7 @@
       </c>
       <c r="Y187" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z187" t="inlineStr">
@@ -21615,7 +21615,7 @@
       </c>
       <c r="Y188" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z188" t="inlineStr">
@@ -21700,7 +21700,7 @@
       </c>
       <c r="Y189" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z189" t="inlineStr">
@@ -21785,7 +21785,7 @@
       </c>
       <c r="Y190" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z190" t="inlineStr">
@@ -21870,7 +21870,7 @@
       </c>
       <c r="Y191" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z191" t="inlineStr">
@@ -21930,7 +21930,7 @@
       </c>
       <c r="Y192" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z192" t="inlineStr">
@@ -22020,7 +22020,7 @@
       </c>
       <c r="Y193" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z193" t="inlineStr">
@@ -22105,7 +22105,7 @@
       </c>
       <c r="Y194" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z194" t="inlineStr">
@@ -22165,7 +22165,7 @@
       </c>
       <c r="Y195" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z195" t="inlineStr">
@@ -22215,7 +22215,7 @@
       </c>
       <c r="Y196" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z196" t="inlineStr">
@@ -22275,7 +22275,7 @@
       </c>
       <c r="Y197" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z197" t="inlineStr">
@@ -22365,7 +22365,7 @@
       </c>
       <c r="Y198" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z198" t="inlineStr">
@@ -22450,7 +22450,7 @@
       </c>
       <c r="Y199" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z199" t="inlineStr">
@@ -22535,7 +22535,7 @@
       </c>
       <c r="Y200" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z200" t="inlineStr">
@@ -22620,7 +22620,7 @@
       </c>
       <c r="Y201" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -22700,7 +22700,7 @@
       </c>
       <c r="Y202" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z202" t="inlineStr">
@@ -22760,7 +22760,7 @@
       </c>
       <c r="Y203" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -22800,7 +22800,7 @@
       </c>
       <c r="Y204" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z204" t="inlineStr">
@@ -22890,7 +22890,7 @@
       </c>
       <c r="Y205" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -22970,7 +22970,7 @@
       </c>
       <c r="Y206" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -23045,7 +23045,7 @@
       </c>
       <c r="Y207" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z207" t="inlineStr">
@@ -23130,7 +23130,7 @@
       </c>
       <c r="Y208" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z208" t="inlineStr">
@@ -23215,7 +23215,7 @@
       </c>
       <c r="Y209" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z209" t="inlineStr">
@@ -23300,7 +23300,7 @@
       </c>
       <c r="Y210" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z210" t="inlineStr">
@@ -23390,7 +23390,7 @@
       </c>
       <c r="Y211" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z211" t="inlineStr">
@@ -23450,7 +23450,7 @@
       </c>
       <c r="Y212" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z212" t="inlineStr">
@@ -23535,7 +23535,7 @@
       </c>
       <c r="Y213" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z213" t="inlineStr">
@@ -23625,7 +23625,7 @@
       </c>
       <c r="Y214" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z214" t="inlineStr">
@@ -23685,7 +23685,7 @@
       </c>
       <c r="Y215" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -23735,7 +23735,7 @@
       </c>
       <c r="Y216" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z216" t="inlineStr">
@@ -23820,7 +23820,7 @@
       </c>
       <c r="Y217" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z217" t="inlineStr">
@@ -23880,7 +23880,7 @@
       </c>
       <c r="Y218" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z218" t="inlineStr">
@@ -23965,7 +23965,7 @@
       </c>
       <c r="Y219" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z219" t="inlineStr">
@@ -24055,7 +24055,7 @@
       </c>
       <c r="Y220" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z220" t="inlineStr">
@@ -24145,7 +24145,7 @@
       </c>
       <c r="Y221" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z221" t="inlineStr">
@@ -24235,7 +24235,7 @@
       </c>
       <c r="Y222" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -24310,7 +24310,7 @@
       </c>
       <c r="Y223" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z223" t="inlineStr">
@@ -24370,7 +24370,7 @@
       </c>
       <c r="Y224" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -24420,7 +24420,7 @@
       </c>
       <c r="Y225" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z225" t="inlineStr">
@@ -24480,7 +24480,7 @@
       </c>
       <c r="Y226" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -24560,7 +24560,7 @@
       </c>
       <c r="Y227" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z227" t="inlineStr">
@@ -24645,7 +24645,7 @@
       </c>
       <c r="Y228" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z228" t="inlineStr">
@@ -24705,7 +24705,7 @@
       </c>
       <c r="Y229" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z229" t="inlineStr">
@@ -24765,7 +24765,7 @@
       </c>
       <c r="Y230" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -24845,7 +24845,7 @@
       </c>
       <c r="Y231" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z231" t="inlineStr">
@@ -24935,7 +24935,7 @@
       </c>
       <c r="Y232" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z232" t="inlineStr">
@@ -25015,7 +25015,7 @@
       </c>
       <c r="Y233" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z233" t="inlineStr">
@@ -25095,7 +25095,7 @@
       </c>
       <c r="Y234" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z234" t="inlineStr">
@@ -25175,7 +25175,7 @@
       </c>
       <c r="Y235" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z235" t="inlineStr">
@@ -25260,7 +25260,7 @@
       </c>
       <c r="Y236" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="Z236" t="inlineStr">
@@ -25350,7 +25350,7 @@
       </c>
       <c r="Y237" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -25430,7 +25430,7 @@
       </c>
       <c r="Y238" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -25510,7 +25510,7 @@
       </c>
       <c r="Y239" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -25590,7 +25590,7 @@
       </c>
       <c r="Y240" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -25670,7 +25670,7 @@
       </c>
       <c r="Y241" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -25750,7 +25750,7 @@
       </c>
       <c r="Y242" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -25830,7 +25830,7 @@
       </c>
       <c r="Y243" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -25910,7 +25910,7 @@
       </c>
       <c r="Y244" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -25990,7 +25990,7 @@
       </c>
       <c r="Y245" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26070,7 +26070,7 @@
       </c>
       <c r="Y246" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26150,7 +26150,7 @@
       </c>
       <c r="Y247" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26230,7 +26230,7 @@
       </c>
       <c r="Y248" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26310,7 +26310,7 @@
       </c>
       <c r="Y249" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26390,7 +26390,7 @@
       </c>
       <c r="Y250" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26470,7 +26470,7 @@
       </c>
       <c r="Y251" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26550,7 +26550,7 @@
       </c>
       <c r="Y252" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26630,7 +26630,7 @@
       </c>
       <c r="Y253" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26710,7 +26710,7 @@
       </c>
       <c r="Y254" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26790,7 +26790,7 @@
       </c>
       <c r="Y255" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26870,7 +26870,7 @@
       </c>
       <c r="Y256" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -26950,7 +26950,7 @@
       </c>
       <c r="Y257" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27030,7 +27030,7 @@
       </c>
       <c r="Y258" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27110,7 +27110,7 @@
       </c>
       <c r="Y259" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27190,7 +27190,7 @@
       </c>
       <c r="Y260" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27270,7 +27270,7 @@
       </c>
       <c r="Y261" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27350,7 +27350,7 @@
       </c>
       <c r="Y262" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27430,7 +27430,7 @@
       </c>
       <c r="Y263" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27510,7 +27510,7 @@
       </c>
       <c r="Y264" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27590,7 +27590,7 @@
       </c>
       <c r="Y265" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27670,7 +27670,7 @@
       </c>
       <c r="Y266" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27750,7 +27750,7 @@
       </c>
       <c r="Y267" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27830,7 +27830,7 @@
       </c>
       <c r="Y268" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27910,7 +27910,7 @@
       </c>
       <c r="Y269" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -27990,7 +27990,7 @@
       </c>
       <c r="Y270" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28070,7 +28070,7 @@
       </c>
       <c r="Y271" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28150,7 +28150,7 @@
       </c>
       <c r="Y272" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28230,7 +28230,7 @@
       </c>
       <c r="Y273" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28310,7 +28310,7 @@
       </c>
       <c r="Y274" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28390,7 +28390,7 @@
       </c>
       <c r="Y275" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28470,7 +28470,7 @@
       </c>
       <c r="Y276" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28550,7 +28550,7 @@
       </c>
       <c r="Y277" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28630,7 +28630,7 @@
       </c>
       <c r="Y278" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28710,7 +28710,7 @@
       </c>
       <c r="Y279" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28790,7 +28790,7 @@
       </c>
       <c r="Y280" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28870,7 +28870,7 @@
       </c>
       <c r="Y281" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -28950,7 +28950,7 @@
       </c>
       <c r="Y282" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29030,7 +29030,7 @@
       </c>
       <c r="Y283" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29110,7 +29110,7 @@
       </c>
       <c r="Y284" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29190,7 +29190,7 @@
       </c>
       <c r="Y285" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29270,7 +29270,7 @@
       </c>
       <c r="Y286" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29350,7 +29350,7 @@
       </c>
       <c r="Y287" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29430,7 +29430,7 @@
       </c>
       <c r="Y288" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29510,7 +29510,7 @@
       </c>
       <c r="Y289" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29590,7 +29590,7 @@
       </c>
       <c r="Y290" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29670,7 +29670,7 @@
       </c>
       <c r="Y291" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29750,7 +29750,7 @@
       </c>
       <c r="Y292" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29830,7 +29830,7 @@
       </c>
       <c r="Y293" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29910,7 +29910,7 @@
       </c>
       <c r="Y294" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -29990,7 +29990,7 @@
       </c>
       <c r="Y295" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30070,7 +30070,7 @@
       </c>
       <c r="Y296" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30150,7 +30150,7 @@
       </c>
       <c r="Y297" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30230,7 +30230,7 @@
       </c>
       <c r="Y298" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30310,7 +30310,7 @@
       </c>
       <c r="Y299" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30390,7 +30390,7 @@
       </c>
       <c r="Y300" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30470,7 +30470,7 @@
       </c>
       <c r="Y301" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30550,7 +30550,7 @@
       </c>
       <c r="Y302" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30630,7 +30630,7 @@
       </c>
       <c r="Y303" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30710,7 +30710,7 @@
       </c>
       <c r="Y304" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30790,7 +30790,7 @@
       </c>
       <c r="Y305" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30870,7 +30870,7 @@
       </c>
       <c r="Y306" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -30950,7 +30950,7 @@
       </c>
       <c r="Y307" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31030,7 +31030,7 @@
       </c>
       <c r="Y308" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31110,7 +31110,7 @@
       </c>
       <c r="Y309" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31190,7 +31190,7 @@
       </c>
       <c r="Y310" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31270,7 +31270,7 @@
       </c>
       <c r="Y311" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31350,7 +31350,7 @@
       </c>
       <c r="Y312" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31430,7 +31430,7 @@
       </c>
       <c r="Y313" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31510,7 +31510,7 @@
       </c>
       <c r="Y314" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31590,7 +31590,7 @@
       </c>
       <c r="Y315" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31670,7 +31670,7 @@
       </c>
       <c r="Y316" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31750,7 +31750,7 @@
       </c>
       <c r="Y317" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31830,7 +31830,7 @@
       </c>
       <c r="Y318" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31910,7 +31910,7 @@
       </c>
       <c r="Y319" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -31990,7 +31990,7 @@
       </c>
       <c r="Y320" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32070,7 +32070,7 @@
       </c>
       <c r="Y321" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32150,7 +32150,7 @@
       </c>
       <c r="Y322" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32230,7 +32230,7 @@
       </c>
       <c r="Y323" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32310,7 +32310,7 @@
       </c>
       <c r="Y324" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32390,7 +32390,7 @@
       </c>
       <c r="Y325" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32470,7 +32470,7 @@
       </c>
       <c r="Y326" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32550,7 +32550,7 @@
       </c>
       <c r="Y327" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32630,7 +32630,7 @@
       </c>
       <c r="Y328" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32710,7 +32710,7 @@
       </c>
       <c r="Y329" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32790,7 +32790,7 @@
       </c>
       <c r="Y330" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32870,7 +32870,7 @@
       </c>
       <c r="Y331" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -32950,7 +32950,7 @@
       </c>
       <c r="Y332" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33030,7 +33030,7 @@
       </c>
       <c r="Y333" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33105,7 +33105,7 @@
       </c>
       <c r="Y334" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33185,7 +33185,7 @@
       </c>
       <c r="Y335" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33265,7 +33265,7 @@
       </c>
       <c r="Y336" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33345,7 +33345,7 @@
       </c>
       <c r="Y337" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33425,7 +33425,7 @@
       </c>
       <c r="Y338" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33505,7 +33505,7 @@
       </c>
       <c r="Y339" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33585,7 +33585,7 @@
       </c>
       <c r="Y340" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33665,7 +33665,7 @@
       </c>
       <c r="Y341" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33745,7 +33745,7 @@
       </c>
       <c r="Y342" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33825,7 +33825,7 @@
       </c>
       <c r="Y343" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33900,7 +33900,7 @@
       </c>
       <c r="Y344" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -33980,7 +33980,7 @@
       </c>
       <c r="Y345" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34055,7 +34055,7 @@
       </c>
       <c r="Y346" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34130,7 +34130,7 @@
       </c>
       <c r="Y347" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34205,7 +34205,7 @@
       </c>
       <c r="Y348" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34285,7 +34285,7 @@
       </c>
       <c r="Y349" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34360,7 +34360,7 @@
       </c>
       <c r="Y350" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34435,7 +34435,7 @@
       </c>
       <c r="Y351" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34510,7 +34510,7 @@
       </c>
       <c r="Y352" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34590,7 +34590,7 @@
       </c>
       <c r="Y353" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34665,7 +34665,7 @@
       </c>
       <c r="Y354" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34745,7 +34745,7 @@
       </c>
       <c r="Y355" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34820,7 +34820,7 @@
       </c>
       <c r="Y356" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34895,7 +34895,7 @@
       </c>
       <c r="Y357" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -34975,7 +34975,7 @@
       </c>
       <c r="Y358" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35050,7 +35050,7 @@
       </c>
       <c r="Y359" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35125,7 +35125,7 @@
       </c>
       <c r="Y360" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35205,7 +35205,7 @@
       </c>
       <c r="Y361" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35285,7 +35285,7 @@
       </c>
       <c r="Y362" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35365,7 +35365,7 @@
       </c>
       <c r="Y363" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35440,7 +35440,7 @@
       </c>
       <c r="Y364" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35520,7 +35520,7 @@
       </c>
       <c r="Y365" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35595,7 +35595,7 @@
       </c>
       <c r="Y366" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35670,7 +35670,7 @@
       </c>
       <c r="Y367" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35750,7 +35750,7 @@
       </c>
       <c r="Y368" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35825,7 +35825,7 @@
       </c>
       <c r="Y369" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35905,7 +35905,7 @@
       </c>
       <c r="Y370" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -35985,7 +35985,7 @@
       </c>
       <c r="Y371" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36060,7 +36060,7 @@
       </c>
       <c r="Y372" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36140,7 +36140,7 @@
       </c>
       <c r="Y373" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36220,7 +36220,7 @@
       </c>
       <c r="Y374" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36295,7 +36295,7 @@
       </c>
       <c r="Y375" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36375,7 +36375,7 @@
       </c>
       <c r="Y376" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36455,7 +36455,7 @@
       </c>
       <c r="Y377" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36530,7 +36530,7 @@
       </c>
       <c r="Y378" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36605,7 +36605,7 @@
       </c>
       <c r="Y379" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36685,7 +36685,7 @@
       </c>
       <c r="Y380" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36765,7 +36765,7 @@
       </c>
       <c r="Y381" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36840,7 +36840,7 @@
       </c>
       <c r="Y382" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36915,7 +36915,7 @@
       </c>
       <c r="Y383" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -36995,7 +36995,7 @@
       </c>
       <c r="Y384" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37075,7 +37075,7 @@
       </c>
       <c r="Y385" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37150,7 +37150,7 @@
       </c>
       <c r="Y386" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37230,7 +37230,7 @@
       </c>
       <c r="Y387" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37305,7 +37305,7 @@
       </c>
       <c r="Y388" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37380,7 +37380,7 @@
       </c>
       <c r="Y389" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37455,7 +37455,7 @@
       </c>
       <c r="Y390" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37535,7 +37535,7 @@
       </c>
       <c r="Y391" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37610,7 +37610,7 @@
       </c>
       <c r="Y392" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37690,7 +37690,7 @@
       </c>
       <c r="Y393" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37765,7 +37765,7 @@
       </c>
       <c r="Y394" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37840,7 +37840,7 @@
       </c>
       <c r="Y395" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -37920,7 +37920,7 @@
       </c>
       <c r="Y396" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38000,7 +38000,7 @@
       </c>
       <c r="Y397" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38080,7 +38080,7 @@
       </c>
       <c r="Y398" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38160,7 +38160,7 @@
       </c>
       <c r="Y399" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38235,7 +38235,7 @@
       </c>
       <c r="Y400" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38315,7 +38315,7 @@
       </c>
       <c r="Y401" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38390,7 +38390,7 @@
       </c>
       <c r="Y402" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38465,7 +38465,7 @@
       </c>
       <c r="Y403" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38540,7 +38540,7 @@
       </c>
       <c r="Y404" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38620,7 +38620,7 @@
       </c>
       <c r="Y405" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38700,7 +38700,7 @@
       </c>
       <c r="Y406" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38780,7 +38780,7 @@
       </c>
       <c r="Y407" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38855,7 +38855,7 @@
       </c>
       <c r="Y408" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -38930,7 +38930,7 @@
       </c>
       <c r="Y409" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39010,7 +39010,7 @@
       </c>
       <c r="Y410" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39085,7 +39085,7 @@
       </c>
       <c r="Y411" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39165,7 +39165,7 @@
       </c>
       <c r="Y412" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39245,7 +39245,7 @@
       </c>
       <c r="Y413" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39325,7 +39325,7 @@
       </c>
       <c r="Y414" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39400,7 +39400,7 @@
       </c>
       <c r="Y415" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39480,7 +39480,7 @@
       </c>
       <c r="Y416" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39555,7 +39555,7 @@
       </c>
       <c r="Y417" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39630,7 +39630,7 @@
       </c>
       <c r="Y418" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39705,7 +39705,7 @@
       </c>
       <c r="Y419" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39780,7 +39780,7 @@
       </c>
       <c r="Y420" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39860,7 +39860,7 @@
       </c>
       <c r="Y421" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -39935,7 +39935,7 @@
       </c>
       <c r="Y422" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40015,7 +40015,7 @@
       </c>
       <c r="Y423" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40090,7 +40090,7 @@
       </c>
       <c r="Y424" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40170,7 +40170,7 @@
       </c>
       <c r="Y425" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40245,7 +40245,7 @@
       </c>
       <c r="Y426" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40325,7 +40325,7 @@
       </c>
       <c r="Y427" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40405,7 +40405,7 @@
       </c>
       <c r="Y428" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40480,7 +40480,7 @@
       </c>
       <c r="Y429" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40560,7 +40560,7 @@
       </c>
       <c r="Y430" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40635,7 +40635,7 @@
       </c>
       <c r="Y431" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40715,7 +40715,7 @@
       </c>
       <c r="Y432" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40790,7 +40790,7 @@
       </c>
       <c r="Y433" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40870,7 +40870,7 @@
       </c>
       <c r="Y434" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -40945,7 +40945,7 @@
       </c>
       <c r="Y435" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41025,7 +41025,7 @@
       </c>
       <c r="Y436" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41100,7 +41100,7 @@
       </c>
       <c r="Y437" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41180,7 +41180,7 @@
       </c>
       <c r="Y438" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41255,7 +41255,7 @@
       </c>
       <c r="Y439" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41335,7 +41335,7 @@
       </c>
       <c r="Y440" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41410,7 +41410,7 @@
       </c>
       <c r="Y441" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41485,7 +41485,7 @@
       </c>
       <c r="Y442" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41560,7 +41560,7 @@
       </c>
       <c r="Y443" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41640,7 +41640,7 @@
       </c>
       <c r="Y444" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41720,7 +41720,7 @@
       </c>
       <c r="Y445" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41800,7 +41800,7 @@
       </c>
       <c r="Y446" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41880,7 +41880,7 @@
       </c>
       <c r="Y447" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -41960,7 +41960,7 @@
       </c>
       <c r="Y448" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42040,7 +42040,7 @@
       </c>
       <c r="Y449" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42120,7 +42120,7 @@
       </c>
       <c r="Y450" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42200,7 +42200,7 @@
       </c>
       <c r="Y451" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42280,7 +42280,7 @@
       </c>
       <c r="Y452" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42360,7 +42360,7 @@
       </c>
       <c r="Y453" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42440,7 +42440,7 @@
       </c>
       <c r="Y454" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42520,7 +42520,7 @@
       </c>
       <c r="Y455" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42600,7 +42600,7 @@
       </c>
       <c r="Y456" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42680,7 +42680,7 @@
       </c>
       <c r="Y457" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42760,7 +42760,7 @@
       </c>
       <c r="Y458" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42840,7 +42840,7 @@
       </c>
       <c r="Y459" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42920,7 +42920,7 @@
       </c>
       <c r="Y460" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -42995,7 +42995,7 @@
       </c>
       <c r="Y461" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43075,7 +43075,7 @@
       </c>
       <c r="Y462" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43155,7 +43155,7 @@
       </c>
       <c r="Y463" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43230,7 +43230,7 @@
       </c>
       <c r="Y464" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43305,7 +43305,7 @@
       </c>
       <c r="Y465" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43380,7 +43380,7 @@
       </c>
       <c r="Y466" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43460,7 +43460,7 @@
       </c>
       <c r="Y467" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43540,7 +43540,7 @@
       </c>
       <c r="Y468" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43620,7 +43620,7 @@
       </c>
       <c r="Y469" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43695,7 +43695,7 @@
       </c>
       <c r="Y470" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43775,7 +43775,7 @@
       </c>
       <c r="Y471" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43855,7 +43855,7 @@
       </c>
       <c r="Y472" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -43935,7 +43935,7 @@
       </c>
       <c r="Y473" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44010,7 +44010,7 @@
       </c>
       <c r="Y474" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44085,7 +44085,7 @@
       </c>
       <c r="Y475" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44145,7 +44145,7 @@
       </c>
       <c r="Y476" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44225,7 +44225,7 @@
       </c>
       <c r="Y477" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44300,7 +44300,7 @@
       </c>
       <c r="Y478" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44375,7 +44375,7 @@
       </c>
       <c r="Y479" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44450,7 +44450,7 @@
       </c>
       <c r="Y480" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44525,7 +44525,7 @@
       </c>
       <c r="Y481" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44600,7 +44600,7 @@
       </c>
       <c r="Y482" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44675,7 +44675,7 @@
       </c>
       <c r="Y483" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44755,7 +44755,7 @@
       </c>
       <c r="Y484" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44830,7 +44830,7 @@
       </c>
       <c r="Y485" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44905,7 +44905,7 @@
       </c>
       <c r="Y486" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -44965,7 +44965,7 @@
       </c>
       <c r="Y487" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45040,7 +45040,7 @@
       </c>
       <c r="Y488" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45120,7 +45120,7 @@
       </c>
       <c r="Y489" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45200,7 +45200,7 @@
       </c>
       <c r="Y490" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45275,7 +45275,7 @@
       </c>
       <c r="Y491" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45355,7 +45355,7 @@
       </c>
       <c r="Y492" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45430,7 +45430,7 @@
       </c>
       <c r="Y493" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45505,7 +45505,7 @@
       </c>
       <c r="Y494" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45580,7 +45580,7 @@
       </c>
       <c r="Y495" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45660,7 +45660,7 @@
       </c>
       <c r="Y496" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45735,7 +45735,7 @@
       </c>
       <c r="Y497" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45815,7 +45815,7 @@
       </c>
       <c r="Y498" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45890,7 +45890,7 @@
       </c>
       <c r="Y499" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -45970,7 +45970,7 @@
       </c>
       <c r="Y500" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46045,7 +46045,7 @@
       </c>
       <c r="Y501" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46125,7 +46125,7 @@
       </c>
       <c r="Y502" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46205,7 +46205,7 @@
       </c>
       <c r="Y503" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46285,7 +46285,7 @@
       </c>
       <c r="Y504" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46365,7 +46365,7 @@
       </c>
       <c r="Y505" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46440,7 +46440,7 @@
       </c>
       <c r="Y506" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46515,7 +46515,7 @@
       </c>
       <c r="Y507" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46590,7 +46590,7 @@
       </c>
       <c r="Y508" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46665,7 +46665,7 @@
       </c>
       <c r="Y509" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46745,7 +46745,7 @@
       </c>
       <c r="Y510" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46825,7 +46825,7 @@
       </c>
       <c r="Y511" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46905,7 +46905,7 @@
       </c>
       <c r="Y512" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -46980,7 +46980,7 @@
       </c>
       <c r="Y513" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47055,7 +47055,7 @@
       </c>
       <c r="Y514" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47135,7 +47135,7 @@
       </c>
       <c r="Y515" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47210,7 +47210,7 @@
       </c>
       <c r="Y516" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47290,7 +47290,7 @@
       </c>
       <c r="Y517" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47370,7 +47370,7 @@
       </c>
       <c r="Y518" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47450,7 +47450,7 @@
       </c>
       <c r="Y519" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47525,7 +47525,7 @@
       </c>
       <c r="Y520" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47605,7 +47605,7 @@
       </c>
       <c r="Y521" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47680,7 +47680,7 @@
       </c>
       <c r="Y522" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47760,7 +47760,7 @@
       </c>
       <c r="Y523" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47835,7 +47835,7 @@
       </c>
       <c r="Y524" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47915,7 +47915,7 @@
       </c>
       <c r="Y525" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -47995,7 +47995,7 @@
       </c>
       <c r="Y526" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48070,7 +48070,7 @@
       </c>
       <c r="Y527" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48145,7 +48145,7 @@
       </c>
       <c r="Y528" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48220,7 +48220,7 @@
       </c>
       <c r="Y529" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48295,7 +48295,7 @@
       </c>
       <c r="Y530" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48370,7 +48370,7 @@
       </c>
       <c r="Y531" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48445,7 +48445,7 @@
       </c>
       <c r="Y532" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48520,7 +48520,7 @@
       </c>
       <c r="Y533" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48595,7 +48595,7 @@
       </c>
       <c r="Y534" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48670,7 +48670,7 @@
       </c>
       <c r="Y535" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48745,7 +48745,7 @@
       </c>
       <c r="Y536" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48820,7 +48820,7 @@
       </c>
       <c r="Y537" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48895,7 +48895,7 @@
       </c>
       <c r="Y538" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -48970,7 +48970,7 @@
       </c>
       <c r="Y539" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49045,7 +49045,7 @@
       </c>
       <c r="Y540" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49105,7 +49105,7 @@
       </c>
       <c r="Y541" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49180,7 +49180,7 @@
       </c>
       <c r="Y542" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49255,7 +49255,7 @@
       </c>
       <c r="Y543" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49330,7 +49330,7 @@
       </c>
       <c r="Y544" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49405,7 +49405,7 @@
       </c>
       <c r="Y545" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49485,7 +49485,7 @@
       </c>
       <c r="Y546" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49560,7 +49560,7 @@
       </c>
       <c r="Y547" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49635,7 +49635,7 @@
       </c>
       <c r="Y548" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49715,7 +49715,7 @@
       </c>
       <c r="Y549" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49775,7 +49775,7 @@
       </c>
       <c r="Y550" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49855,7 +49855,7 @@
       </c>
       <c r="Y551" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -49930,7 +49930,7 @@
       </c>
       <c r="Y552" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -50005,7 +50005,7 @@
       </c>
       <c r="Y553" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -50085,7 +50085,7 @@
       </c>
       <c r="Y554" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -50165,7 +50165,7 @@
       </c>
       <c r="Y555" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -50240,7 +50240,7 @@
       </c>
       <c r="Y556" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -50315,7 +50315,7 @@
       </c>
       <c r="Y557" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-29 17:06:51)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -33963,6 +33963,11 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S345" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="T345" t="inlineStr">
         <is>
           <t>902890316</t>
@@ -39923,6 +39928,11 @@
           <t>Kollej</t>
         </is>
       </c>
+      <c r="S422" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
       <c r="V422" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -40078,6 +40088,16 @@
           <t>Kollej</t>
         </is>
       </c>
+      <c r="S424" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="T424" t="inlineStr">
+        <is>
+          <t>883823800 / 914510727</t>
+        </is>
+      </c>
       <c r="V424" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -43218,6 +43238,16 @@
           <t>Kollej</t>
         </is>
       </c>
+      <c r="S464" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="T464" t="inlineStr">
+        <is>
+          <t>886341692 / 973868774</t>
+        </is>
+      </c>
       <c r="V464" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44073,6 +44103,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S475" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="T475" t="inlineStr">
+        <is>
+          <t>910702172 / 90008906</t>
+        </is>
+      </c>
       <c r="V475" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44133,6 +44173,31 @@
           <t>27.04.1997</t>
         </is>
       </c>
+      <c r="O476" t="inlineStr">
+        <is>
+          <t>K 6071373</t>
+        </is>
+      </c>
+      <c r="Q476" t="inlineStr">
+        <is>
+          <t>Kitob sanoat va xizmat ko'rsatish kasb-hunar kolleji</t>
+        </is>
+      </c>
+      <c r="R476" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="S476" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="T476" t="inlineStr">
+        <is>
+          <t>332079255 / 973816690</t>
+        </is>
+      </c>
       <c r="V476" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44288,6 +44353,16 @@
           <t>Kollej</t>
         </is>
       </c>
+      <c r="S478" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="T478" t="inlineStr">
+        <is>
+          <t>973512025 / 905170817</t>
+        </is>
+      </c>
       <c r="V478" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44893,6 +44968,16 @@
           <t>Kollej</t>
         </is>
       </c>
+      <c r="S486" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="T486" t="inlineStr">
+        <is>
+          <t>906792298 / 912245369</t>
+        </is>
+      </c>
       <c r="V486" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -44953,6 +45038,31 @@
           <t>31.01.1996</t>
         </is>
       </c>
+      <c r="O487" t="inlineStr">
+        <is>
+          <t>K 6070161</t>
+        </is>
+      </c>
+      <c r="Q487" t="inlineStr">
+        <is>
+          <t>Kasb-hunar kolleji</t>
+        </is>
+      </c>
+      <c r="R487" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="S487" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="T487" t="inlineStr">
+        <is>
+          <t>500303196 / 973841481</t>
+        </is>
+      </c>
       <c r="V487" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -45493,6 +45603,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S494" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="T494" t="inlineStr">
+        <is>
+          <t>951880530</t>
+        </is>
+      </c>
       <c r="V494" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48358,6 +48478,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S531" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="T531" t="inlineStr">
+        <is>
+          <t>912185816</t>
+        </is>
+      </c>
       <c r="V531" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48433,6 +48563,16 @@
           <t>Kollej</t>
         </is>
       </c>
+      <c r="S532" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="T532" t="inlineStr">
+        <is>
+          <t>915979292 / 501118920</t>
+        </is>
+      </c>
       <c r="V532" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48508,6 +48648,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S533" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="T533" t="inlineStr">
+        <is>
+          <t>505109703 / 873227515</t>
+        </is>
+      </c>
       <c r="V533" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48583,6 +48733,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S534" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="T534" t="inlineStr">
+        <is>
+          <t>886323773 / 914708493</t>
+        </is>
+      </c>
       <c r="V534" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -48733,6 +48893,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S536" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="T536" t="inlineStr">
+        <is>
+          <t>918198931</t>
+        </is>
+      </c>
       <c r="V536" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49093,6 +49263,31 @@
           <t>20.03.2002</t>
         </is>
       </c>
+      <c r="O541" t="inlineStr">
+        <is>
+          <t>D 0094389</t>
+        </is>
+      </c>
+      <c r="Q541" t="inlineStr">
+        <is>
+          <t>Sharisabz tuman Chorshanbe agrosanoat kasb-hunar kolleji</t>
+        </is>
+      </c>
+      <c r="R541" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="S541" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="T541" t="inlineStr">
+        <is>
+          <t>975895253 / 873225253</t>
+        </is>
+      </c>
       <c r="V541" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49243,6 +49438,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S543" t="inlineStr">
+        <is>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="T543" t="inlineStr">
+        <is>
+          <t>881309088 / 935831388</t>
+        </is>
+      </c>
       <c r="V543" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49318,6 +49523,16 @@
           <t>Kollej</t>
         </is>
       </c>
+      <c r="S544" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="T544" t="inlineStr">
+        <is>
+          <t>918142047 / 888040008</t>
+        </is>
+      </c>
       <c r="V544" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49393,6 +49608,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S545" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="T545" t="inlineStr">
+        <is>
+          <t>913211605</t>
+        </is>
+      </c>
       <c r="V545" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49623,6 +49848,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S548" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="T548" t="inlineStr">
+        <is>
+          <t>883862204 / 887789709</t>
+        </is>
+      </c>
       <c r="V548" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49763,6 +49998,21 @@
           <t>19.07.1995</t>
         </is>
       </c>
+      <c r="Q550" t="inlineStr">
+        <is>
+          <t>Kasb-hunar kolleji</t>
+        </is>
+      </c>
+      <c r="R550" t="inlineStr">
+        <is>
+          <t>Kollej</t>
+        </is>
+      </c>
+      <c r="T550" t="inlineStr">
+        <is>
+          <t>870350795 / 971997200</t>
+        </is>
+      </c>
       <c r="V550" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49918,6 +50168,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S552" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T552" t="inlineStr">
+        <is>
+          <t>916402192 / 883807881</t>
+        </is>
+      </c>
       <c r="V552" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -49993,6 +50253,16 @@
           <t>Umumiy o'rta maktab</t>
         </is>
       </c>
+      <c r="S553" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="T553" t="inlineStr">
+        <is>
+          <t>919634966 / 908988509</t>
+        </is>
+      </c>
       <c r="V553" t="inlineStr">
         <is>
           <t>2025-2026 kontingenti: 2-kurs</t>
@@ -50226,6 +50496,16 @@
       <c r="R556" t="inlineStr">
         <is>
           <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="S556" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="T556" t="inlineStr">
+        <is>
+          <t>777350767 / 973550702</t>
         </is>
       </c>
       <c r="V556" t="inlineStr">

</xml_diff>

<commit_message>
Bazaga kiritilganligi (KIRITILDI/KIRITILMAGAN) tasdiqlash turi qo'shildi
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA557"/>
+  <dimension ref="A1:AB557"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -555,6 +555,11 @@
           <t>Buyruq sanasi</t>
         </is>
       </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Bazaga kiritilganligi</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">

</xml_diff>

<commit_message>
25-16 guruhiga 3 nafar yangi talaba qo'shildi (ID-karta rasmlari bilan)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB557"/>
+  <dimension ref="A1:AB560"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50604,6 +50604,276 @@
         </is>
       </c>
     </row>
+    <row r="558">
+      <c r="A558" t="n">
+        <v>557</v>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Abdiraimova Shahzoda</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>Dilshod qizi</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>Abdiraimova Shahzoda Dilshod qizi</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>ABDIRAIMOVA SHAHZODA DILSHOD QIZI</t>
+        </is>
+      </c>
+      <c r="J558" t="inlineStr">
+        <is>
+          <t>AD8711360</t>
+        </is>
+      </c>
+      <c r="K558" t="inlineStr">
+        <is>
+          <t>61511075720098</t>
+        </is>
+      </c>
+      <c r="L558" t="inlineStr">
+        <is>
+          <t>20.09.2024</t>
+        </is>
+      </c>
+      <c r="M558" t="inlineStr">
+        <is>
+          <t>15.11.2007</t>
+        </is>
+      </c>
+      <c r="Q558" t="inlineStr">
+        <is>
+          <t>Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="R558" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="U558" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V558" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs</t>
+        </is>
+      </c>
+      <c r="W558" t="inlineStr">
+        <is>
+          <t>25-16</t>
+        </is>
+      </c>
+      <c r="X558" t="inlineStr">
+        <is>
+          <t>MOS (TO'LIQ)</t>
+        </is>
+      </c>
+      <c r="Y558" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="AB558" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="n">
+        <v>558</v>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Hayitova Xolida</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>Asad qizi</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>Hayitova Xolida Asad qizi</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>HAYITOVA XOLIDA ASAD QIZI</t>
+        </is>
+      </c>
+      <c r="J559" t="inlineStr">
+        <is>
+          <t>AD5343254</t>
+        </is>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>61112065720083</t>
+        </is>
+      </c>
+      <c r="L559" t="inlineStr">
+        <is>
+          <t>06.12.2023</t>
+        </is>
+      </c>
+      <c r="M559" t="inlineStr">
+        <is>
+          <t>11.12.2006</t>
+        </is>
+      </c>
+      <c r="Q559" t="inlineStr">
+        <is>
+          <t>Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="R559" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="U559" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V559" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs</t>
+        </is>
+      </c>
+      <c r="W559" t="inlineStr">
+        <is>
+          <t>25-16</t>
+        </is>
+      </c>
+      <c r="X559" t="inlineStr">
+        <is>
+          <t>MOS (TO'LIQ)</t>
+        </is>
+      </c>
+      <c r="Y559" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="AB559" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="n">
+        <v>559</v>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Shog'dorova Marjona</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi</t>
+        </is>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>Eshtemir qizi</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>Shog'dorova Marjona Eshtemir qizi</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>SHOG'DOROVA MARJONA ESHTEMIR QIZI</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>AD9143185</t>
+        </is>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>63006075720080</t>
+        </is>
+      </c>
+      <c r="L560" t="inlineStr">
+        <is>
+          <t>24.10.2024</t>
+        </is>
+      </c>
+      <c r="M560" t="inlineStr">
+        <is>
+          <t>30.06.2007</t>
+        </is>
+      </c>
+      <c r="Q560" t="inlineStr">
+        <is>
+          <t>Chiroqchi tumani</t>
+        </is>
+      </c>
+      <c r="R560" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="U560" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V560" t="inlineStr">
+        <is>
+          <t>2025-2026 kontingenti: 2-kurs</t>
+        </is>
+      </c>
+      <c r="W560" t="inlineStr">
+        <is>
+          <t>25-16</t>
+        </is>
+      </c>
+      <c r="X560" t="inlineStr">
+        <is>
+          <t>MOS (TO'LIQ)</t>
+        </is>
+      </c>
+      <c r="Y560" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="AB560" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-30 16:19:50)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB560"/>
+  <dimension ref="A1:AB563"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50874,6 +50874,327 @@
         </is>
       </c>
     </row>
+    <row r="561">
+      <c r="A561" t="n">
+        <v>560</v>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Tursunmurodova Diyora</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr"/>
+      <c r="F561" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>Jasur qizi</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>Tursunmurodova Diyora Jasur qizi</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>AD9513015</t>
+        </is>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>61609075680011</t>
+        </is>
+      </c>
+      <c r="L561" t="inlineStr">
+        <is>
+          <t>21.11.2024</t>
+        </is>
+      </c>
+      <c r="M561" t="inlineStr">
+        <is>
+          <t>16.09.2007</t>
+        </is>
+      </c>
+      <c r="N561" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O561" t="inlineStr">
+        <is>
+          <t>UM 03274052</t>
+        </is>
+      </c>
+      <c r="P561" t="inlineStr"/>
+      <c r="Q561" t="inlineStr">
+        <is>
+          <t>Qashqadaryo viloyati, Kitob tumani 25-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R561" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S561" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="T561" t="inlineStr">
+        <is>
+          <t>887611310</t>
+        </is>
+      </c>
+      <c r="U561" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W561" t="inlineStr">
+        <is>
+          <t>26-03</t>
+        </is>
+      </c>
+      <c r="Y561" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB561" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="n">
+        <v>561</v>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Rashidova Shaxzoda</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E562" t="inlineStr"/>
+      <c r="F562" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>Suyun qizi</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>Rashidova Shaxzoda Suyun qizi</t>
+        </is>
+      </c>
+      <c r="J562" t="inlineStr">
+        <is>
+          <t>AD6348784</t>
+        </is>
+      </c>
+      <c r="K562" t="inlineStr">
+        <is>
+          <t>61408075590081</t>
+        </is>
+      </c>
+      <c r="L562" t="inlineStr">
+        <is>
+          <t>04.03.2024</t>
+        </is>
+      </c>
+      <c r="M562" t="inlineStr">
+        <is>
+          <t>14.08.2007</t>
+        </is>
+      </c>
+      <c r="N562" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O562" t="inlineStr">
+        <is>
+          <t>UM 02171747</t>
+        </is>
+      </c>
+      <c r="P562" t="inlineStr"/>
+      <c r="Q562" t="inlineStr">
+        <is>
+          <t>Sesoni umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R562" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S562" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T562" t="inlineStr">
+        <is>
+          <t>94-806-00-14</t>
+        </is>
+      </c>
+      <c r="U562" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W562" t="inlineStr">
+        <is>
+          <t>26-02</t>
+        </is>
+      </c>
+      <c r="Y562" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB562" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="n">
+        <v>562</v>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Rashidova Shaxzoda</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr"/>
+      <c r="F563" t="inlineStr">
+        <is>
+          <t>30.09.2026</t>
+        </is>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>Suyun qizi</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>Rashidova Shaxzoda Suyun qizi</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>AD6348784</t>
+        </is>
+      </c>
+      <c r="K563" t="inlineStr">
+        <is>
+          <t>61408075590081</t>
+        </is>
+      </c>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>04.03.2024</t>
+        </is>
+      </c>
+      <c r="M563" t="inlineStr">
+        <is>
+          <t>14.08.2007</t>
+        </is>
+      </c>
+      <c r="N563" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O563" t="inlineStr">
+        <is>
+          <t>UM 02171747</t>
+        </is>
+      </c>
+      <c r="P563" t="inlineStr"/>
+      <c r="Q563" t="inlineStr">
+        <is>
+          <t>5-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R563" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S563" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="T563" t="inlineStr">
+        <is>
+          <t>94-806-00-14</t>
+        </is>
+      </c>
+      <c r="U563" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W563" t="inlineStr">
+        <is>
+          <t>24-15</t>
+        </is>
+      </c>
+      <c r="Y563" t="inlineStr">
+        <is>
+          <t>KUTILMOQDA</t>
+        </is>
+      </c>
+      <c r="AB563" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-30 16:21:27)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB563"/>
+  <dimension ref="A1:AB562"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50893,7 +50893,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E561" t="inlineStr"/>
       <c r="F561" t="inlineStr">
         <is>
           <t>30.09.2026</t>
@@ -50939,7 +50938,6 @@
           <t>UM 03274052</t>
         </is>
       </c>
-      <c r="P561" t="inlineStr"/>
       <c r="Q561" t="inlineStr">
         <is>
           <t>Qashqadaryo viloyati, Kitob tumani 25-sonli umumiy o'rta ta'lim maktabini</t>
@@ -51000,7 +50998,6 @@
           <t>To'lov qildi</t>
         </is>
       </c>
-      <c r="E562" t="inlineStr"/>
       <c r="F562" t="inlineStr">
         <is>
           <t>30.09.2026</t>
@@ -51046,10 +51043,9 @@
           <t>UM 02171747</t>
         </is>
       </c>
-      <c r="P562" t="inlineStr"/>
       <c r="Q562" t="inlineStr">
         <is>
-          <t>Sesoni umumiy o'rta ta'lim maktabini</t>
+          <t>5-sonli umumiy o'rta ta'lim maktabini</t>
         </is>
       </c>
       <c r="R562" t="inlineStr">
@@ -51074,7 +51070,7 @@
       </c>
       <c r="W562" t="inlineStr">
         <is>
-          <t>26-02</t>
+          <t>24-15</t>
         </is>
       </c>
       <c r="Y562" t="inlineStr">
@@ -51083,113 +51079,6 @@
         </is>
       </c>
       <c r="AB562" t="inlineStr">
-        <is>
-          <t>KIRITILDI</t>
-        </is>
-      </c>
-    </row>
-    <row r="563">
-      <c r="A563" t="n">
-        <v>562</v>
-      </c>
-      <c r="B563" t="inlineStr">
-        <is>
-          <t>Rashidova Shaxzoda</t>
-        </is>
-      </c>
-      <c r="C563" t="inlineStr">
-        <is>
-          <t>Hamshiralik ishi - 3 yillik</t>
-        </is>
-      </c>
-      <c r="D563" t="inlineStr">
-        <is>
-          <t>To'lov qildi</t>
-        </is>
-      </c>
-      <c r="E563" t="inlineStr"/>
-      <c r="F563" t="inlineStr">
-        <is>
-          <t>30.09.2026</t>
-        </is>
-      </c>
-      <c r="G563" t="inlineStr">
-        <is>
-          <t>Suyun qizi</t>
-        </is>
-      </c>
-      <c r="H563" t="inlineStr">
-        <is>
-          <t>Rashidova Shaxzoda Suyun qizi</t>
-        </is>
-      </c>
-      <c r="J563" t="inlineStr">
-        <is>
-          <t>AD6348784</t>
-        </is>
-      </c>
-      <c r="K563" t="inlineStr">
-        <is>
-          <t>61408075590081</t>
-        </is>
-      </c>
-      <c r="L563" t="inlineStr">
-        <is>
-          <t>04.03.2024</t>
-        </is>
-      </c>
-      <c r="M563" t="inlineStr">
-        <is>
-          <t>14.08.2007</t>
-        </is>
-      </c>
-      <c r="N563" t="inlineStr">
-        <is>
-          <t>Mavjud</t>
-        </is>
-      </c>
-      <c r="O563" t="inlineStr">
-        <is>
-          <t>UM 02171747</t>
-        </is>
-      </c>
-      <c r="P563" t="inlineStr"/>
-      <c r="Q563" t="inlineStr">
-        <is>
-          <t>5-sonli umumiy o'rta ta'lim maktabini</t>
-        </is>
-      </c>
-      <c r="R563" t="inlineStr">
-        <is>
-          <t>Shahodatnoma</t>
-        </is>
-      </c>
-      <c r="S563" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="T563" t="inlineStr">
-        <is>
-          <t>94-806-00-14</t>
-        </is>
-      </c>
-      <c r="U563" t="inlineStr">
-        <is>
-          <t>TOPILDI</t>
-        </is>
-      </c>
-      <c r="W563" t="inlineStr">
-        <is>
-          <t>24-15</t>
-        </is>
-      </c>
-      <c r="Y563" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
-        </is>
-      </c>
-      <c r="AB563" t="inlineStr">
         <is>
           <t>KIRITILDI</t>
         </is>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-30 16:24:15)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -676,6 +676,11 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-30 16:47:26)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -39955,7 +39955,7 @@
       </c>
       <c r="Y422" t="inlineStr">
         <is>
-          <t>TASDIQLANDI</t>
+          <t>KUTILMOQDA</t>
         </is>
       </c>
     </row>
@@ -40120,7 +40120,7 @@
       </c>
       <c r="Y424" t="inlineStr">
         <is>
-          <t>TASDIQLANDI</t>
+          <t>KUTILMOQDA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-30 16:53:05)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB562"/>
+  <dimension ref="A1:AB563"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51089,6 +51089,104 @@
         </is>
       </c>
     </row>
+    <row r="563">
+      <c r="A563" t="n">
+        <v>562</v>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Zaripova Setora</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="F563" t="inlineStr"/>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>Zuxriddin qizi</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>Zaripova Setora Zuxriddin qizi</t>
+        </is>
+      </c>
+      <c r="J563" t="inlineStr">
+        <is>
+          <t>AD8594631</t>
+        </is>
+      </c>
+      <c r="K563" t="inlineStr">
+        <is>
+          <t>60609075730014</t>
+        </is>
+      </c>
+      <c r="L563" t="inlineStr">
+        <is>
+          <t>12.09.2024</t>
+        </is>
+      </c>
+      <c r="M563" t="inlineStr">
+        <is>
+          <t>06.09.2007</t>
+        </is>
+      </c>
+      <c r="N563" t="inlineStr"/>
+      <c r="O563" t="inlineStr">
+        <is>
+          <t>UM 03299021</t>
+        </is>
+      </c>
+      <c r="P563" t="inlineStr"/>
+      <c r="Q563" t="inlineStr">
+        <is>
+          <t>1-sonli umumiy o'rta ta'lim maktabini</t>
+        </is>
+      </c>
+      <c r="R563" t="inlineStr">
+        <is>
+          <t>Umumiy o'rta maktab</t>
+        </is>
+      </c>
+      <c r="S563" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="T563" t="inlineStr">
+        <is>
+          <t>773893666 / 606090757</t>
+        </is>
+      </c>
+      <c r="U563" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="V563" t="inlineStr">
+        <is>
+          <t>AI orqali tahlil qilinib qo'shildi</t>
+        </is>
+      </c>
+      <c r="W563" t="inlineStr">
+        <is>
+          <t>25-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-30 16:53:44)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -51080,7 +51080,7 @@
       </c>
       <c r="Y562" t="inlineStr">
         <is>
-          <t>KUTILMOQDA</t>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
       <c r="AB562" t="inlineStr">
@@ -51113,7 +51113,6 @@
           <t>226</t>
         </is>
       </c>
-      <c r="F563" t="inlineStr"/>
       <c r="G563" t="inlineStr">
         <is>
           <t>Zuxriddin qizi</t>
@@ -51144,13 +51143,11 @@
           <t>06.09.2007</t>
         </is>
       </c>
-      <c r="N563" t="inlineStr"/>
       <c r="O563" t="inlineStr">
         <is>
           <t>UM 03299021</t>
         </is>
       </c>
-      <c r="P563" t="inlineStr"/>
       <c r="Q563" t="inlineStr">
         <is>
           <t>1-sonli umumiy o'rta ta'lim maktabini</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-09-30 16:54:55)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -51183,6 +51183,16 @@
           <t>25-17</t>
         </is>
       </c>
+      <c r="Y563" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="AB563" t="inlineStr">
+        <is>
+          <t>KIRITILMAGAN</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-07 08:16:06)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -2321,8 +2321,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -4663,8 +4661,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z34" t="inlineStr"/>
-      <c r="AA34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -9608,8 +9604,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z74" t="inlineStr"/>
-      <c r="AA74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -22391,7 +22385,7 @@
       </c>
       <c r="W177" t="inlineStr">
         <is>
-          <t>26-06</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="Y177" t="inlineStr">
@@ -22401,12 +22395,12 @@
       </c>
       <c r="Z177" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA177" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>06.10.2026</t>
         </is>
       </c>
     </row>
@@ -24479,8 +24473,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z201" t="inlineStr"/>
-      <c r="AA201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -24621,8 +24613,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z203" t="inlineStr"/>
-      <c r="AA203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -24753,8 +24743,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z205" t="inlineStr"/>
-      <c r="AA205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -24835,8 +24823,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z206" t="inlineStr"/>
-      <c r="AA206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -25552,8 +25538,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z215" t="inlineStr"/>
-      <c r="AA215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -26099,8 +26083,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z222" t="inlineStr"/>
-      <c r="AA222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -26236,8 +26218,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z224" t="inlineStr"/>
-      <c r="AA224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -26348,8 +26328,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z226" t="inlineStr"/>
-      <c r="AA226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -26635,8 +26613,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z230" t="inlineStr"/>
-      <c r="AA230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -27227,8 +27203,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z237" t="inlineStr"/>
-      <c r="AA237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -27314,8 +27288,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z238" t="inlineStr"/>
-      <c r="AA238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -27401,8 +27373,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z239" t="inlineStr"/>
-      <c r="AA239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -27488,8 +27458,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z240" t="inlineStr"/>
-      <c r="AA240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -27570,8 +27538,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z241" t="inlineStr"/>
-      <c r="AA241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -27652,8 +27618,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z242" t="inlineStr"/>
-      <c r="AA242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -27734,8 +27698,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z243" t="inlineStr"/>
-      <c r="AA243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -27816,8 +27778,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z244" t="inlineStr"/>
-      <c r="AA244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -27903,8 +27863,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z245" t="inlineStr"/>
-      <c r="AA245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -27985,8 +27943,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z246" t="inlineStr"/>
-      <c r="AA246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -28067,8 +28023,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z247" t="inlineStr"/>
-      <c r="AA247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -28149,8 +28103,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z248" t="inlineStr"/>
-      <c r="AA248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -28231,8 +28183,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z249" t="inlineStr"/>
-      <c r="AA249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -28313,8 +28263,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z250" t="inlineStr"/>
-      <c r="AA250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -28395,8 +28343,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z251" t="inlineStr"/>
-      <c r="AA251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -28482,8 +28428,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z252" t="inlineStr"/>
-      <c r="AA252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -28569,8 +28513,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z253" t="inlineStr"/>
-      <c r="AA253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -28656,8 +28598,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z254" t="inlineStr"/>
-      <c r="AA254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -28738,8 +28678,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z255" t="inlineStr"/>
-      <c r="AA255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -28825,8 +28763,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z256" t="inlineStr"/>
-      <c r="AA256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -28907,8 +28843,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z257" t="inlineStr"/>
-      <c r="AA257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -28989,8 +28923,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z258" t="inlineStr"/>
-      <c r="AA258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -29071,8 +29003,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z259" t="inlineStr"/>
-      <c r="AA259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -29153,8 +29083,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z260" t="inlineStr"/>
-      <c r="AA260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -29235,8 +29163,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z261" t="inlineStr"/>
-      <c r="AA261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -29317,8 +29243,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z262" t="inlineStr"/>
-      <c r="AA262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -29399,8 +29323,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z263" t="inlineStr"/>
-      <c r="AA263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -29481,8 +29403,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z264" t="inlineStr"/>
-      <c r="AA264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -29563,8 +29483,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z265" t="inlineStr"/>
-      <c r="AA265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -29645,8 +29563,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z266" t="inlineStr"/>
-      <c r="AA266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -29727,8 +29643,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z267" t="inlineStr"/>
-      <c r="AA267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -29809,8 +29723,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z268" t="inlineStr"/>
-      <c r="AA268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -29891,8 +29803,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z269" t="inlineStr"/>
-      <c r="AA269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -29973,8 +29883,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z270" t="inlineStr"/>
-      <c r="AA270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -30060,8 +29968,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z271" t="inlineStr"/>
-      <c r="AA271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -30142,8 +30048,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z272" t="inlineStr"/>
-      <c r="AA272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -30229,8 +30133,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z273" t="inlineStr"/>
-      <c r="AA273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -30316,8 +30218,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z274" t="inlineStr"/>
-      <c r="AA274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -30403,8 +30303,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z275" t="inlineStr"/>
-      <c r="AA275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -30485,8 +30383,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z276" t="inlineStr"/>
-      <c r="AA276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -30572,8 +30468,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z277" t="inlineStr"/>
-      <c r="AA277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -30654,8 +30548,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z278" t="inlineStr"/>
-      <c r="AA278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -30736,8 +30628,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z279" t="inlineStr"/>
-      <c r="AA279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -30818,8 +30708,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z280" t="inlineStr"/>
-      <c r="AA280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -30900,8 +30788,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z281" t="inlineStr"/>
-      <c r="AA281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -30982,8 +30868,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z282" t="inlineStr"/>
-      <c r="AA282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -31064,8 +30948,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z283" t="inlineStr"/>
-      <c r="AA283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -31146,8 +31028,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z284" t="inlineStr"/>
-      <c r="AA284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -31228,8 +31108,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z285" t="inlineStr"/>
-      <c r="AA285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -31310,8 +31188,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z286" t="inlineStr"/>
-      <c r="AA286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -31392,8 +31268,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z287" t="inlineStr"/>
-      <c r="AA287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -31474,8 +31348,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z288" t="inlineStr"/>
-      <c r="AA288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -31561,8 +31433,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z289" t="inlineStr"/>
-      <c r="AA289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -31643,8 +31513,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z290" t="inlineStr"/>
-      <c r="AA290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -31725,8 +31593,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z291" t="inlineStr"/>
-      <c r="AA291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -31807,8 +31673,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z292" t="inlineStr"/>
-      <c r="AA292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -31894,8 +31758,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z293" t="inlineStr"/>
-      <c r="AA293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -31981,8 +31843,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z294" t="inlineStr"/>
-      <c r="AA294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -32063,8 +31923,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z295" t="inlineStr"/>
-      <c r="AA295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -32145,8 +32003,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z296" t="inlineStr"/>
-      <c r="AA296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -32227,8 +32083,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z297" t="inlineStr"/>
-      <c r="AA297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -32309,8 +32163,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z298" t="inlineStr"/>
-      <c r="AA298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -32391,8 +32243,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z299" t="inlineStr"/>
-      <c r="AA299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -32473,8 +32323,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z300" t="inlineStr"/>
-      <c r="AA300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -32560,8 +32408,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z301" t="inlineStr"/>
-      <c r="AA301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -32647,8 +32493,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z302" t="inlineStr"/>
-      <c r="AA302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -32729,8 +32573,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z303" t="inlineStr"/>
-      <c r="AA303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -32811,8 +32653,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z304" t="inlineStr"/>
-      <c r="AA304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -32893,8 +32733,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z305" t="inlineStr"/>
-      <c r="AA305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -32980,8 +32818,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z306" t="inlineStr"/>
-      <c r="AA306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -33062,8 +32898,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z307" t="inlineStr"/>
-      <c r="AA307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -33144,8 +32978,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z308" t="inlineStr"/>
-      <c r="AA308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -33226,8 +33058,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z309" t="inlineStr"/>
-      <c r="AA309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -33308,8 +33138,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z310" t="inlineStr"/>
-      <c r="AA310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -33390,8 +33218,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z311" t="inlineStr"/>
-      <c r="AA311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -33477,8 +33303,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z312" t="inlineStr"/>
-      <c r="AA312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -33559,8 +33383,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z313" t="inlineStr"/>
-      <c r="AA313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -33641,8 +33463,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z314" t="inlineStr"/>
-      <c r="AA314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -33723,8 +33543,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z315" t="inlineStr"/>
-      <c r="AA315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -33810,8 +33628,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z316" t="inlineStr"/>
-      <c r="AA316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -33892,8 +33708,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z317" t="inlineStr"/>
-      <c r="AA317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -33974,8 +33788,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z318" t="inlineStr"/>
-      <c r="AA318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -34061,8 +33873,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z319" t="inlineStr"/>
-      <c r="AA319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -34143,8 +33953,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z320" t="inlineStr"/>
-      <c r="AA320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -34225,8 +34033,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z321" t="inlineStr"/>
-      <c r="AA321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -34307,8 +34113,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z322" t="inlineStr"/>
-      <c r="AA322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -34389,8 +34193,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z323" t="inlineStr"/>
-      <c r="AA323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -34471,8 +34273,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z324" t="inlineStr"/>
-      <c r="AA324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -34553,8 +34353,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z325" t="inlineStr"/>
-      <c r="AA325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -34635,8 +34433,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z326" t="inlineStr"/>
-      <c r="AA326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -34717,8 +34513,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z327" t="inlineStr"/>
-      <c r="AA327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -34799,8 +34593,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z328" t="inlineStr"/>
-      <c r="AA328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="n">
@@ -34881,8 +34673,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z329" t="inlineStr"/>
-      <c r="AA329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -34968,8 +34758,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z330" t="inlineStr"/>
-      <c r="AA330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -35050,8 +34838,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z331" t="inlineStr"/>
-      <c r="AA331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -35132,8 +34918,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z332" t="inlineStr"/>
-      <c r="AA332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -35214,8 +34998,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z333" t="inlineStr"/>
-      <c r="AA333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -35291,8 +35073,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z334" t="inlineStr"/>
-      <c r="AA334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -35378,8 +35158,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z335" t="inlineStr"/>
-      <c r="AA335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -35460,8 +35238,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z336" t="inlineStr"/>
-      <c r="AA336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -35547,8 +35323,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z337" t="inlineStr"/>
-      <c r="AA337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -35629,8 +35403,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z338" t="inlineStr"/>
-      <c r="AA338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -35711,8 +35483,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z339" t="inlineStr"/>
-      <c r="AA339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -35793,8 +35563,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z340" t="inlineStr"/>
-      <c r="AA340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -35875,8 +35643,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z341" t="inlineStr"/>
-      <c r="AA341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -35957,8 +35723,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z342" t="inlineStr"/>
-      <c r="AA342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -36039,8 +35803,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z343" t="inlineStr"/>
-      <c r="AA343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -36116,8 +35878,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z344" t="inlineStr"/>
-      <c r="AA344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -36203,8 +35963,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z345" t="inlineStr"/>
-      <c r="AA345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -36280,8 +36038,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z346" t="inlineStr"/>
-      <c r="AA346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="n">
@@ -36357,8 +36113,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z347" t="inlineStr"/>
-      <c r="AA347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -36439,8 +36193,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z348" t="inlineStr"/>
-      <c r="AA348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -36521,8 +36273,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z349" t="inlineStr"/>
-      <c r="AA349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -36598,8 +36348,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z350" t="inlineStr"/>
-      <c r="AA350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="n">
@@ -36675,8 +36423,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z351" t="inlineStr"/>
-      <c r="AA351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -36752,8 +36498,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z352" t="inlineStr"/>
-      <c r="AA352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="n">
@@ -36834,8 +36578,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z353" t="inlineStr"/>
-      <c r="AA353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -36911,8 +36653,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z354" t="inlineStr"/>
-      <c r="AA354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -36993,8 +36733,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z355" t="inlineStr"/>
-      <c r="AA355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -37070,8 +36808,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z356" t="inlineStr"/>
-      <c r="AA356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -37147,8 +36883,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z357" t="inlineStr"/>
-      <c r="AA357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -37229,8 +36963,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z358" t="inlineStr"/>
-      <c r="AA358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -37306,8 +37038,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z359" t="inlineStr"/>
-      <c r="AA359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -37383,8 +37113,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z360" t="inlineStr"/>
-      <c r="AA360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -37465,8 +37193,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z361" t="inlineStr"/>
-      <c r="AA361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -37547,8 +37273,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z362" t="inlineStr"/>
-      <c r="AA362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="n">
@@ -37634,8 +37358,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z363" t="inlineStr"/>
-      <c r="AA363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -37711,8 +37433,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z364" t="inlineStr"/>
-      <c r="AA364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -37798,8 +37518,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z365" t="inlineStr"/>
-      <c r="AA365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -37875,8 +37593,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z366" t="inlineStr"/>
-      <c r="AA366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="n">
@@ -37952,8 +37668,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z367" t="inlineStr"/>
-      <c r="AA367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -38034,8 +37748,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z368" t="inlineStr"/>
-      <c r="AA368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -38111,8 +37823,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z369" t="inlineStr"/>
-      <c r="AA369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="n">
@@ -38193,8 +37903,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z370" t="inlineStr"/>
-      <c r="AA370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="n">
@@ -38280,8 +37988,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z371" t="inlineStr"/>
-      <c r="AA371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="n">
@@ -38357,8 +38063,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z372" t="inlineStr"/>
-      <c r="AA372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="n">
@@ -38439,8 +38143,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z373" t="inlineStr"/>
-      <c r="AA373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="n">
@@ -38521,8 +38223,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z374" t="inlineStr"/>
-      <c r="AA374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="n">
@@ -38598,8 +38298,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z375" t="inlineStr"/>
-      <c r="AA375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="n">
@@ -38685,8 +38383,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z376" t="inlineStr"/>
-      <c r="AA376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="n">
@@ -38767,8 +38463,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z377" t="inlineStr"/>
-      <c r="AA377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="n">
@@ -38849,8 +38543,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z378" t="inlineStr"/>
-      <c r="AA378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="n">
@@ -38926,8 +38618,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z379" t="inlineStr"/>
-      <c r="AA379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="n">
@@ -39013,8 +38703,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z380" t="inlineStr"/>
-      <c r="AA380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="n">
@@ -39095,8 +38783,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z381" t="inlineStr"/>
-      <c r="AA381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="n">
@@ -39172,8 +38858,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z382" t="inlineStr"/>
-      <c r="AA382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="n">
@@ -39249,8 +38933,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z383" t="inlineStr"/>
-      <c r="AA383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="n">
@@ -39331,8 +39013,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z384" t="inlineStr"/>
-      <c r="AA384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="n">
@@ -39413,8 +39093,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z385" t="inlineStr"/>
-      <c r="AA385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="n">
@@ -39490,8 +39168,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z386" t="inlineStr"/>
-      <c r="AA386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="n">
@@ -39572,8 +39248,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z387" t="inlineStr"/>
-      <c r="AA387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="n">
@@ -39654,8 +39328,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z388" t="inlineStr"/>
-      <c r="AA388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="n">
@@ -39731,8 +39403,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z389" t="inlineStr"/>
-      <c r="AA389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="n">
@@ -39808,8 +39478,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z390" t="inlineStr"/>
-      <c r="AA390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="n">
@@ -39890,8 +39558,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z391" t="inlineStr"/>
-      <c r="AA391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="n">
@@ -39967,8 +39633,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z392" t="inlineStr"/>
-      <c r="AA392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="n">
@@ -40049,8 +39713,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z393" t="inlineStr"/>
-      <c r="AA393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="n">
@@ -40126,8 +39788,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z394" t="inlineStr"/>
-      <c r="AA394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="n">
@@ -40203,8 +39863,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z395" t="inlineStr"/>
-      <c r="AA395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="n">
@@ -40285,8 +39943,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z396" t="inlineStr"/>
-      <c r="AA396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="n">
@@ -40367,8 +40023,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z397" t="inlineStr"/>
-      <c r="AA397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="n">
@@ -40454,8 +40108,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z398" t="inlineStr"/>
-      <c r="AA398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="n">
@@ -40541,8 +40193,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z399" t="inlineStr"/>
-      <c r="AA399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="n">
@@ -40618,8 +40268,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z400" t="inlineStr"/>
-      <c r="AA400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="n">
@@ -40700,8 +40348,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z401" t="inlineStr"/>
-      <c r="AA401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="n">
@@ -40777,8 +40423,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z402" t="inlineStr"/>
-      <c r="AA402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="n">
@@ -40854,8 +40498,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z403" t="inlineStr"/>
-      <c r="AA403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="n">
@@ -40936,8 +40578,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z404" t="inlineStr"/>
-      <c r="AA404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="n">
@@ -41023,8 +40663,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z405" t="inlineStr"/>
-      <c r="AA405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="n">
@@ -41105,8 +40743,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z406" t="inlineStr"/>
-      <c r="AA406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="n">
@@ -41187,8 +40823,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z407" t="inlineStr"/>
-      <c r="AA407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="n">
@@ -41264,8 +40898,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z408" t="inlineStr"/>
-      <c r="AA408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="n">
@@ -41341,8 +40973,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z409" t="inlineStr"/>
-      <c r="AA409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="n">
@@ -41423,8 +41053,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z410" t="inlineStr"/>
-      <c r="AA410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="n">
@@ -41500,8 +41128,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z411" t="inlineStr"/>
-      <c r="AA411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" t="n">
@@ -41582,8 +41208,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z412" t="inlineStr"/>
-      <c r="AA412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" t="n">
@@ -41664,8 +41288,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z413" t="inlineStr"/>
-      <c r="AA413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="n">
@@ -41751,8 +41373,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z414" t="inlineStr"/>
-      <c r="AA414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="n">
@@ -41828,8 +41448,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z415" t="inlineStr"/>
-      <c r="AA415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="n">
@@ -41910,8 +41528,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z416" t="inlineStr"/>
-      <c r="AA416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="n">
@@ -41987,8 +41603,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z417" t="inlineStr"/>
-      <c r="AA417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="n">
@@ -42064,8 +41678,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z418" t="inlineStr"/>
-      <c r="AA418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="n">
@@ -42141,8 +41753,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z419" t="inlineStr"/>
-      <c r="AA419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="n">
@@ -42218,8 +41828,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z420" t="inlineStr"/>
-      <c r="AA420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="n">
@@ -42300,8 +41908,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z421" t="inlineStr"/>
-      <c r="AA421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="n">
@@ -42382,8 +41988,6 @@
           <t>KUTILMOQDA</t>
         </is>
       </c>
-      <c r="Z422" t="inlineStr"/>
-      <c r="AA422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="n">
@@ -42469,8 +42073,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z423" t="inlineStr"/>
-      <c r="AA423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="n">
@@ -42556,8 +42158,6 @@
           <t>KUTILMOQDA</t>
         </is>
       </c>
-      <c r="Z424" t="inlineStr"/>
-      <c r="AA424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" t="n">
@@ -42638,8 +42238,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z425" t="inlineStr"/>
-      <c r="AA425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" t="n">
@@ -42720,8 +42318,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z426" t="inlineStr"/>
-      <c r="AA426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="n">
@@ -42802,8 +42398,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z427" t="inlineStr"/>
-      <c r="AA427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="n">
@@ -42889,8 +42483,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z428" t="inlineStr"/>
-      <c r="AA428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="n">
@@ -42971,8 +42563,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z429" t="inlineStr"/>
-      <c r="AA429" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" t="n">
@@ -43053,8 +42643,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z430" t="inlineStr"/>
-      <c r="AA430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="n">
@@ -43130,8 +42718,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z431" t="inlineStr"/>
-      <c r="AA431" t="inlineStr"/>
     </row>
     <row r="432">
       <c r="A432" t="n">
@@ -43217,8 +42803,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z432" t="inlineStr"/>
-      <c r="AA432" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" t="n">
@@ -43294,8 +42878,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z433" t="inlineStr"/>
-      <c r="AA433" t="inlineStr"/>
     </row>
     <row r="434">
       <c r="A434" t="n">
@@ -43376,8 +42958,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z434" t="inlineStr"/>
-      <c r="AA434" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" t="n">
@@ -43453,8 +43033,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z435" t="inlineStr"/>
-      <c r="AA435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="n">
@@ -43540,8 +43118,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z436" t="inlineStr"/>
-      <c r="AA436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" t="n">
@@ -43622,8 +43198,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z437" t="inlineStr"/>
-      <c r="AA437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="n">
@@ -43704,8 +43278,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z438" t="inlineStr"/>
-      <c r="AA438" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" t="n">
@@ -43781,8 +43353,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z439" t="inlineStr"/>
-      <c r="AA439" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" t="n">
@@ -43863,8 +43433,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z440" t="inlineStr"/>
-      <c r="AA440" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" t="n">
@@ -43940,8 +43508,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z441" t="inlineStr"/>
-      <c r="AA441" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" t="n">
@@ -44017,8 +43583,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z442" t="inlineStr"/>
-      <c r="AA442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" t="n">
@@ -44099,8 +43663,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z443" t="inlineStr"/>
-      <c r="AA443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" t="n">
@@ -44181,8 +43743,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z444" t="inlineStr"/>
-      <c r="AA444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" t="n">
@@ -44258,8 +43818,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z445" t="inlineStr"/>
-      <c r="AA445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="n">
@@ -44345,8 +43903,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z446" t="inlineStr"/>
-      <c r="AA446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="n">
@@ -44427,8 +43983,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z447" t="inlineStr"/>
-      <c r="AA447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" t="n">
@@ -44514,8 +44068,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z448" t="inlineStr"/>
-      <c r="AA448" t="inlineStr"/>
     </row>
     <row r="449">
       <c r="A449" t="n">
@@ -44596,8 +44148,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z449" t="inlineStr"/>
-      <c r="AA449" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" t="n">
@@ -44678,8 +44228,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z450" t="inlineStr"/>
-      <c r="AA450" t="inlineStr"/>
     </row>
     <row r="451">
       <c r="A451" t="n">
@@ -44765,8 +44313,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z451" t="inlineStr"/>
-      <c r="AA451" t="inlineStr"/>
     </row>
     <row r="452">
       <c r="A452" t="n">
@@ -44942,8 +44488,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z453" t="inlineStr"/>
-      <c r="AA453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="n">
@@ -45029,8 +44573,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z454" t="inlineStr"/>
-      <c r="AA454" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" t="n">
@@ -45116,8 +44658,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z455" t="inlineStr"/>
-      <c r="AA455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="n">
@@ -45198,8 +44738,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z456" t="inlineStr"/>
-      <c r="AA456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" t="n">
@@ -45280,8 +44818,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z457" t="inlineStr"/>
-      <c r="AA457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" t="n">
@@ -45362,8 +44898,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z458" t="inlineStr"/>
-      <c r="AA458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" t="n">
@@ -45444,8 +44978,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z459" t="inlineStr"/>
-      <c r="AA459" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" t="n">
@@ -45526,8 +45058,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z460" t="inlineStr"/>
-      <c r="AA460" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" t="n">
@@ -45603,8 +45133,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z461" t="inlineStr"/>
-      <c r="AA461" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" t="n">
@@ -45690,8 +45218,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z462" t="inlineStr"/>
-      <c r="AA462" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" t="n">
@@ -45772,8 +45298,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z463" t="inlineStr"/>
-      <c r="AA463" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" t="n">
@@ -45859,8 +45383,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z464" t="inlineStr"/>
-      <c r="AA464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" t="n">
@@ -45936,8 +45458,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z465" t="inlineStr"/>
-      <c r="AA465" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" t="n">
@@ -46013,8 +45533,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z466" t="inlineStr"/>
-      <c r="AA466" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" t="n">
@@ -46095,8 +45613,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z467" t="inlineStr"/>
-      <c r="AA467" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" t="n">
@@ -46177,8 +45693,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z468" t="inlineStr"/>
-      <c r="AA468" t="inlineStr"/>
     </row>
     <row r="469">
       <c r="A469" t="n">
@@ -46259,8 +45773,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z469" t="inlineStr"/>
-      <c r="AA469" t="inlineStr"/>
     </row>
     <row r="470">
       <c r="A470" t="n">
@@ -46336,8 +45848,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z470" t="inlineStr"/>
-      <c r="AA470" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" t="n">
@@ -46423,8 +45933,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z471" t="inlineStr"/>
-      <c r="AA471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" t="n">
@@ -46510,8 +46018,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z472" t="inlineStr"/>
-      <c r="AA472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" t="n">
@@ -46597,8 +46103,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z473" t="inlineStr"/>
-      <c r="AA473" t="inlineStr"/>
     </row>
     <row r="474">
       <c r="A474" t="n">
@@ -46674,8 +46178,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z474" t="inlineStr"/>
-      <c r="AA474" t="inlineStr"/>
     </row>
     <row r="475">
       <c r="A475" t="n">
@@ -46761,8 +46263,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z475" t="inlineStr"/>
-      <c r="AA475" t="inlineStr"/>
     </row>
     <row r="476">
       <c r="A476" t="n">
@@ -46848,8 +46348,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z476" t="inlineStr"/>
-      <c r="AA476" t="inlineStr"/>
     </row>
     <row r="477">
       <c r="A477" t="n">
@@ -46930,8 +46428,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z477" t="inlineStr"/>
-      <c r="AA477" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" t="n">
@@ -47017,8 +46513,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z478" t="inlineStr"/>
-      <c r="AA478" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" t="n">
@@ -47094,8 +46588,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z479" t="inlineStr"/>
-      <c r="AA479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" t="n">
@@ -47171,8 +46663,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z480" t="inlineStr"/>
-      <c r="AA480" t="inlineStr"/>
     </row>
     <row r="481">
       <c r="A481" t="n">
@@ -47253,8 +46743,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z481" t="inlineStr"/>
-      <c r="AA481" t="inlineStr"/>
     </row>
     <row r="482">
       <c r="A482" t="n">
@@ -47330,8 +46818,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z482" t="inlineStr"/>
-      <c r="AA482" t="inlineStr"/>
     </row>
     <row r="483">
       <c r="A483" t="n">
@@ -47407,8 +46893,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z483" t="inlineStr"/>
-      <c r="AA483" t="inlineStr"/>
     </row>
     <row r="484">
       <c r="A484" t="n">
@@ -47494,8 +46978,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z484" t="inlineStr"/>
-      <c r="AA484" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" t="n">
@@ -47576,8 +47058,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z485" t="inlineStr"/>
-      <c r="AA485" t="inlineStr"/>
     </row>
     <row r="486">
       <c r="A486" t="n">
@@ -47663,8 +47143,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z486" t="inlineStr"/>
-      <c r="AA486" t="inlineStr"/>
     </row>
     <row r="487">
       <c r="A487" t="n">
@@ -47755,8 +47233,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z487" t="inlineStr"/>
-      <c r="AA487" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" t="n">
@@ -47832,8 +47308,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z488" t="inlineStr"/>
-      <c r="AA488" t="inlineStr"/>
     </row>
     <row r="489">
       <c r="A489" t="n">
@@ -47909,8 +47383,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z489" t="inlineStr"/>
-      <c r="AA489" t="inlineStr"/>
     </row>
     <row r="490">
       <c r="A490" t="n">
@@ -47986,8 +47458,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z490" t="inlineStr"/>
-      <c r="AA490" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" t="n">
@@ -48063,8 +47533,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z491" t="inlineStr"/>
-      <c r="AA491" t="inlineStr"/>
     </row>
     <row r="492">
       <c r="A492" t="n">
@@ -48140,8 +47608,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z492" t="inlineStr"/>
-      <c r="AA492" t="inlineStr"/>
     </row>
     <row r="493">
       <c r="A493" t="n">
@@ -48217,8 +47683,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z493" t="inlineStr"/>
-      <c r="AA493" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" t="n">
@@ -48309,8 +47773,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z494" t="inlineStr"/>
-      <c r="AA494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="n">
@@ -48391,8 +47853,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z495" t="inlineStr"/>
-      <c r="AA495" t="inlineStr"/>
     </row>
     <row r="496">
       <c r="A496" t="n">
@@ -48473,8 +47933,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z496" t="inlineStr"/>
-      <c r="AA496" t="inlineStr"/>
     </row>
     <row r="497">
       <c r="A497" t="n">
@@ -48550,8 +48008,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z497" t="inlineStr"/>
-      <c r="AA497" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" t="n">
@@ -48637,8 +48093,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z498" t="inlineStr"/>
-      <c r="AA498" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" t="n">
@@ -48714,8 +48168,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z499" t="inlineStr"/>
-      <c r="AA499" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" t="n">
@@ -48801,8 +48253,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z500" t="inlineStr"/>
-      <c r="AA500" t="inlineStr"/>
     </row>
     <row r="501">
       <c r="A501" t="n">
@@ -48878,8 +48328,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z501" t="inlineStr"/>
-      <c r="AA501" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" t="n">
@@ -48960,8 +48408,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z502" t="inlineStr"/>
-      <c r="AA502" t="inlineStr"/>
     </row>
     <row r="503">
       <c r="A503" t="n">
@@ -49042,8 +48488,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z503" t="inlineStr"/>
-      <c r="AA503" t="inlineStr"/>
     </row>
     <row r="504">
       <c r="A504" t="n">
@@ -49124,8 +48568,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z504" t="inlineStr"/>
-      <c r="AA504" t="inlineStr"/>
     </row>
     <row r="505">
       <c r="A505" t="n">
@@ -49206,8 +48648,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z505" t="inlineStr"/>
-      <c r="AA505" t="inlineStr"/>
     </row>
     <row r="506">
       <c r="A506" t="n">
@@ -49283,8 +48723,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z506" t="inlineStr"/>
-      <c r="AA506" t="inlineStr"/>
     </row>
     <row r="507">
       <c r="A507" t="n">
@@ -49360,8 +48798,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z507" t="inlineStr"/>
-      <c r="AA507" t="inlineStr"/>
     </row>
     <row r="508">
       <c r="A508" t="n">
@@ -49442,8 +48878,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z508" t="inlineStr"/>
-      <c r="AA508" t="inlineStr"/>
     </row>
     <row r="509">
       <c r="A509" t="n">
@@ -49519,8 +48953,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z509" t="inlineStr"/>
-      <c r="AA509" t="inlineStr"/>
     </row>
     <row r="510">
       <c r="A510" t="n">
@@ -49601,8 +49033,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z510" t="inlineStr"/>
-      <c r="AA510" t="inlineStr"/>
     </row>
     <row r="511">
       <c r="A511" t="n">
@@ -49683,8 +49113,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z511" t="inlineStr"/>
-      <c r="AA511" t="inlineStr"/>
     </row>
     <row r="512">
       <c r="A512" t="n">
@@ -49770,8 +49198,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z512" t="inlineStr"/>
-      <c r="AA512" t="inlineStr"/>
     </row>
     <row r="513">
       <c r="A513" t="n">
@@ -49847,8 +49273,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z513" t="inlineStr"/>
-      <c r="AA513" t="inlineStr"/>
     </row>
     <row r="514">
       <c r="A514" t="n">
@@ -49929,8 +49353,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z514" t="inlineStr"/>
-      <c r="AA514" t="inlineStr"/>
     </row>
     <row r="515">
       <c r="A515" t="n">
@@ -50011,8 +49433,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z515" t="inlineStr"/>
-      <c r="AA515" t="inlineStr"/>
     </row>
     <row r="516">
       <c r="A516" t="n">
@@ -50088,8 +49508,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z516" t="inlineStr"/>
-      <c r="AA516" t="inlineStr"/>
     </row>
     <row r="517">
       <c r="A517" t="n">
@@ -50170,8 +49588,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z517" t="inlineStr"/>
-      <c r="AA517" t="inlineStr"/>
     </row>
     <row r="518">
       <c r="A518" t="n">
@@ -50252,8 +49668,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z518" t="inlineStr"/>
-      <c r="AA518" t="inlineStr"/>
     </row>
     <row r="519">
       <c r="A519" t="n">
@@ -50334,8 +49748,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z519" t="inlineStr"/>
-      <c r="AA519" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" t="n">
@@ -50411,8 +49823,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z520" t="inlineStr"/>
-      <c r="AA520" t="inlineStr"/>
     </row>
     <row r="521">
       <c r="A521" t="n">
@@ -50493,8 +49903,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z521" t="inlineStr"/>
-      <c r="AA521" t="inlineStr"/>
     </row>
     <row r="522">
       <c r="A522" t="n">
@@ -50570,8 +49978,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z522" t="inlineStr"/>
-      <c r="AA522" t="inlineStr"/>
     </row>
     <row r="523">
       <c r="A523" t="n">
@@ -50652,8 +50058,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z523" t="inlineStr"/>
-      <c r="AA523" t="inlineStr"/>
     </row>
     <row r="524">
       <c r="A524" t="n">
@@ -50729,8 +50133,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z524" t="inlineStr"/>
-      <c r="AA524" t="inlineStr"/>
     </row>
     <row r="525">
       <c r="A525" t="n">
@@ -50816,8 +50218,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z525" t="inlineStr"/>
-      <c r="AA525" t="inlineStr"/>
     </row>
     <row r="526">
       <c r="A526" t="n">
@@ -50898,8 +50298,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z526" t="inlineStr"/>
-      <c r="AA526" t="inlineStr"/>
     </row>
     <row r="527">
       <c r="A527" t="n">
@@ -50980,8 +50378,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z527" t="inlineStr"/>
-      <c r="AA527" t="inlineStr"/>
     </row>
     <row r="528">
       <c r="A528" t="n">
@@ -51052,8 +50448,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z528" t="inlineStr"/>
-      <c r="AA528" t="inlineStr"/>
     </row>
     <row r="529">
       <c r="A529" t="n">
@@ -51129,8 +50523,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z529" t="inlineStr"/>
-      <c r="AA529" t="inlineStr"/>
     </row>
     <row r="530">
       <c r="A530" t="n">
@@ -51206,8 +50598,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z530" t="inlineStr"/>
-      <c r="AA530" t="inlineStr"/>
     </row>
     <row r="531">
       <c r="A531" t="n">
@@ -51293,8 +50683,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z531" t="inlineStr"/>
-      <c r="AA531" t="inlineStr"/>
     </row>
     <row r="532">
       <c r="A532" t="n">
@@ -51385,8 +50773,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z532" t="inlineStr"/>
-      <c r="AA532" t="inlineStr"/>
     </row>
     <row r="533">
       <c r="A533" t="n">
@@ -51477,8 +50863,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z533" t="inlineStr"/>
-      <c r="AA533" t="inlineStr"/>
     </row>
     <row r="534">
       <c r="A534" t="n">
@@ -51564,8 +50948,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z534" t="inlineStr"/>
-      <c r="AA534" t="inlineStr"/>
     </row>
     <row r="535">
       <c r="A535" t="n">
@@ -51641,8 +51023,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z535" t="inlineStr"/>
-      <c r="AA535" t="inlineStr"/>
     </row>
     <row r="536">
       <c r="A536" t="n">
@@ -51728,8 +51108,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z536" t="inlineStr"/>
-      <c r="AA536" t="inlineStr"/>
     </row>
     <row r="537">
       <c r="A537" t="n">
@@ -51805,8 +51183,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z537" t="inlineStr"/>
-      <c r="AA537" t="inlineStr"/>
     </row>
     <row r="538">
       <c r="A538" t="n">
@@ -51887,8 +51263,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z538" t="inlineStr"/>
-      <c r="AA538" t="inlineStr"/>
     </row>
     <row r="539">
       <c r="A539" t="n">
@@ -51969,8 +51343,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z539" t="inlineStr"/>
-      <c r="AA539" t="inlineStr"/>
     </row>
     <row r="540">
       <c r="A540" t="n">
@@ -52046,8 +51418,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z540" t="inlineStr"/>
-      <c r="AA540" t="inlineStr"/>
     </row>
     <row r="541">
       <c r="A541" t="n">
@@ -52133,8 +51503,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z541" t="inlineStr"/>
-      <c r="AA541" t="inlineStr"/>
     </row>
     <row r="542">
       <c r="A542" t="n">
@@ -52305,8 +51673,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z543" t="inlineStr"/>
-      <c r="AA543" t="inlineStr"/>
     </row>
     <row r="544">
       <c r="A544" t="n">
@@ -52397,8 +51763,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z544" t="inlineStr"/>
-      <c r="AA544" t="inlineStr"/>
     </row>
     <row r="545">
       <c r="A545" t="n">
@@ -52484,8 +51848,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z545" t="inlineStr"/>
-      <c r="AA545" t="inlineStr"/>
     </row>
     <row r="546">
       <c r="A546" t="n">
@@ -52561,8 +51923,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z546" t="inlineStr"/>
-      <c r="AA546" t="inlineStr"/>
     </row>
     <row r="547">
       <c r="A547" t="n">
@@ -52638,8 +51998,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z547" t="inlineStr"/>
-      <c r="AA547" t="inlineStr"/>
     </row>
     <row r="548">
       <c r="A548" t="n">
@@ -52730,8 +52088,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z548" t="inlineStr"/>
-      <c r="AA548" t="inlineStr"/>
     </row>
     <row r="549">
       <c r="A549" t="n">
@@ -52807,8 +52163,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z549" t="inlineStr"/>
-      <c r="AA549" t="inlineStr"/>
     </row>
     <row r="550">
       <c r="A550" t="n">
@@ -52884,8 +52238,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z550" t="inlineStr"/>
-      <c r="AA550" t="inlineStr"/>
     </row>
     <row r="551">
       <c r="A551" t="n">
@@ -52966,8 +52318,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z551" t="inlineStr"/>
-      <c r="AA551" t="inlineStr"/>
     </row>
     <row r="552">
       <c r="A552" t="n">
@@ -53058,8 +52408,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z552" t="inlineStr"/>
-      <c r="AA552" t="inlineStr"/>
     </row>
     <row r="553">
       <c r="A553" t="n">
@@ -53145,8 +52493,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z553" t="inlineStr"/>
-      <c r="AA553" t="inlineStr"/>
     </row>
     <row r="554">
       <c r="A554" t="n">
@@ -53227,8 +52573,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z554" t="inlineStr"/>
-      <c r="AA554" t="inlineStr"/>
     </row>
     <row r="555">
       <c r="A555" t="n">
@@ -53309,8 +52653,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z555" t="inlineStr"/>
-      <c r="AA555" t="inlineStr"/>
     </row>
     <row r="556">
       <c r="A556" t="n">
@@ -53401,8 +52743,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z556" t="inlineStr"/>
-      <c r="AA556" t="inlineStr"/>
     </row>
     <row r="557">
       <c r="A557" t="n">
@@ -53573,8 +52913,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z558" t="inlineStr"/>
-      <c r="AA558" t="inlineStr"/>
       <c r="AB558" t="inlineStr">
         <is>
           <t>KIRITILDI</t>
@@ -53665,8 +53003,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z559" t="inlineStr"/>
-      <c r="AA559" t="inlineStr"/>
       <c r="AB559" t="inlineStr">
         <is>
           <t>KIRITILDI</t>
@@ -53757,8 +53093,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z560" t="inlineStr"/>
-      <c r="AA560" t="inlineStr"/>
       <c r="AB560" t="inlineStr">
         <is>
           <t>KIRITILDI</t>
@@ -53984,8 +53318,6 @@
           <t>TASDIQLANDI</t>
         </is>
       </c>
-      <c r="Z562" t="inlineStr"/>
-      <c r="AA562" t="inlineStr"/>
       <c r="AB562" t="inlineStr">
         <is>
           <t>KIRITILDI</t>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-08 10:50:27)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -39395,12 +39395,22 @@
       </c>
       <c r="W389" t="inlineStr">
         <is>
-          <t>25-17</t>
+          <t>Akademik ta'til olganlar</t>
         </is>
       </c>
       <c r="Y389" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="Z389" t="inlineStr">
+        <is>
+          <t>T-52</t>
+        </is>
+      </c>
+      <c r="AA389" t="inlineStr">
+        <is>
+          <t>05.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-09 13:12:59)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -23005,17 +23005,17 @@
       </c>
       <c r="W183" t="inlineStr">
         <is>
-          <t>26-02</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="Z183" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA183" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>09.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-09 13:13:47)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -22705,7 +22705,7 @@
       </c>
       <c r="W180" t="inlineStr">
         <is>
-          <t>26-02</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="Y180" t="inlineStr">
@@ -22715,12 +22715,12 @@
       </c>
       <c r="Z180" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA180" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>09.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-09 14:29:21)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -37105,12 +37105,22 @@
       </c>
       <c r="W360" t="inlineStr">
         <is>
-          <t>25-16</t>
+          <t>Akademik ta'til olganlar</t>
         </is>
       </c>
       <c r="Y360" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="Z360" t="inlineStr">
+        <is>
+          <t>T-50</t>
+        </is>
+      </c>
+      <c r="AA360" t="inlineStr">
+        <is>
+          <t>02.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-09 16:39:46)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -52830,7 +52830,7 @@
       </c>
       <c r="W557" t="inlineStr">
         <is>
-          <t>25-19</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="Y557" t="inlineStr">
@@ -52840,12 +52840,12 @@
       </c>
       <c r="Z557" t="inlineStr">
         <is>
-          <t>T-28</t>
+          <t>T-53</t>
         </is>
       </c>
       <c r="AA557" t="inlineStr">
         <is>
-          <t>20.03.2026</t>
+          <t>09.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-14 09:47:20)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Toliq_Royxati.xlsx
+++ b/data/Talabalar_Toliq_Royxati.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB563"/>
+  <dimension ref="A1:AB564"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10219,7 +10219,7 @@
       </c>
       <c r="W79" t="inlineStr">
         <is>
-          <t>26-03</t>
+          <t>26-07</t>
         </is>
       </c>
       <c r="X79" t="inlineStr">
@@ -22595,7 +22595,7 @@
       </c>
       <c r="W179" t="inlineStr">
         <is>
-          <t>26-03</t>
+          <t>26-07</t>
         </is>
       </c>
       <c r="Y179" t="inlineStr">
@@ -23105,17 +23105,17 @@
       </c>
       <c r="W184" t="inlineStr">
         <is>
-          <t>26-02</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="Z184" t="inlineStr">
         <is>
-          <t>T-40/2</t>
+          <t>---</t>
         </is>
       </c>
       <c r="AA184" t="inlineStr">
         <is>
-          <t>02.09.2026</t>
+          <t>10.10.2026</t>
         </is>
       </c>
     </row>
@@ -37750,12 +37750,22 @@
       </c>
       <c r="W368" t="inlineStr">
         <is>
-          <t>25-16</t>
+          <t>Talabalar safidan chiqarilganlar</t>
         </is>
       </c>
       <c r="Y368" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="Z368" t="inlineStr">
+        <is>
+          <t>T-54</t>
+        </is>
+      </c>
+      <c r="AA368" t="inlineStr">
+        <is>
+          <t>10.09.2026</t>
         </is>
       </c>
     </row>
@@ -40835,12 +40845,22 @@
       </c>
       <c r="W407" t="inlineStr">
         <is>
-          <t>25-18</t>
+          <t>Akademik ta'til olganlar</t>
         </is>
       </c>
       <c r="Y407" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="Z407" t="inlineStr">
+        <is>
+          <t>T-55</t>
+        </is>
+      </c>
+      <c r="AA407" t="inlineStr">
+        <is>
+          <t>13.10.2026</t>
         </is>
       </c>
     </row>
@@ -41690,12 +41710,22 @@
       </c>
       <c r="W418" t="inlineStr">
         <is>
-          <t>25-18</t>
+          <t>Akademik ta'til olganlar</t>
         </is>
       </c>
       <c r="Y418" t="inlineStr">
         <is>
           <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="Z418" t="inlineStr">
+        <is>
+          <t>T-56</t>
+        </is>
+      </c>
+      <c r="AA418" t="inlineStr">
+        <is>
+          <t>13.10.2026</t>
         </is>
       </c>
     </row>
@@ -53456,6 +53486,113 @@
       <c r="AB563" t="inlineStr">
         <is>
           <t>KIRITILMAGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="n">
+        <v>563</v>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Jumayeva Sabina</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Hamshiralik ishi - 3 yillik</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>To'lov qildi</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>331</t>
+        </is>
+      </c>
+      <c r="F564" t="inlineStr">
+        <is>
+          <t>14.10.2026</t>
+        </is>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>Sobir qizi</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>Jumayeva Sabina Sobir qizi</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>AD9154749</t>
+        </is>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>62411085590063</t>
+        </is>
+      </c>
+      <c r="L564" t="inlineStr">
+        <is>
+          <t>26.10.2024</t>
+        </is>
+      </c>
+      <c r="M564" t="inlineStr">
+        <is>
+          <t>24.11.2008</t>
+        </is>
+      </c>
+      <c r="N564" t="inlineStr">
+        <is>
+          <t>Mavjud</t>
+        </is>
+      </c>
+      <c r="O564" t="inlineStr">
+        <is>
+          <t>UM 03752398</t>
+        </is>
+      </c>
+      <c r="P564" t="inlineStr"/>
+      <c r="Q564" t="inlineStr">
+        <is>
+          <t>13-sonli umumiy o'rta ta'lim maktabi</t>
+        </is>
+      </c>
+      <c r="R564" t="inlineStr">
+        <is>
+          <t>Shahodatnoma</t>
+        </is>
+      </c>
+      <c r="S564" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="T564" t="inlineStr"/>
+      <c r="U564" t="inlineStr">
+        <is>
+          <t>TOPILDI</t>
+        </is>
+      </c>
+      <c r="W564" t="inlineStr">
+        <is>
+          <t>26-03</t>
+        </is>
+      </c>
+      <c r="Y564" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
+        </is>
+      </c>
+      <c r="AB564" t="inlineStr">
+        <is>
+          <t>KIRITILDI</t>
         </is>
       </c>
     </row>

</xml_diff>